<commit_message>
J Block Data Added
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -23215,7 +23215,7 @@
         <v>2263</v>
       </c>
       <c r="B1967" s="2" t="n">
-        <v>745</v>
+        <v>767</v>
       </c>
     </row>
     <row r="1968" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24215,7 +24215,7 @@
         <v>2389</v>
       </c>
       <c r="B2092" s="2" t="n">
-        <v>245</v>
+        <v>705</v>
       </c>
     </row>
     <row r="2093" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
C block list 6 updated
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2449" uniqueCount="2448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2464" uniqueCount="2458">
   <si>
     <t xml:space="preserve">Flat Number</t>
   </si>
@@ -6379,622 +6379,901 @@
     <t xml:space="preserve">J5-1201</t>
   </si>
   <si>
+    <t xml:space="preserve">C1-1703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">426-427</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1203A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-2001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1204A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">532-533</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">519-520</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">565A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">538-539</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">528-529</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1203A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-2003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1203A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">477A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1906</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">442-443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">439-440</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1205A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">448-449</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1203A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">430-431</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-2001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B361</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1745A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1202A</t>
+  </si>
+  <si>
     <t xml:space="preserve">C1-1106</t>
   </si>
   <si>
-    <t xml:space="preserve">C1-1902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1205A</t>
+    <t xml:space="preserve">C5-706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">485-486</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">493-494</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1205A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">558A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">583A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1204A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-2006</t>
   </si>
   <si>
     <t xml:space="preserve">C2-804</t>
   </si>
   <si>
-    <t xml:space="preserve">C2-102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1405</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1406</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-2001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1204A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1504</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-904</t>
+    <t xml:space="preserve">C2-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1204A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">547A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1205A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1103</t>
   </si>
   <si>
     <t xml:space="preserve">C4-1102</t>
   </si>
   <si>
-    <t xml:space="preserve">C4-1904</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1203A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-505</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-706</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1906</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1205A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1405</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-603</t>
+    <t xml:space="preserve">C2-604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">557B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">536-537</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c4-405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c4-804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c3-403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c4-806</t>
   </si>
   <si>
     <t xml:space="preserve">c5-2005</t>
   </si>
   <si>
+    <t xml:space="preserve">c2-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-1802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-1001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-506</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">428-429</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B370B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c4-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-1506</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">532A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-206</t>
+  </si>
+  <si>
     <t xml:space="preserve">C4-1406</t>
   </si>
   <si>
-    <t xml:space="preserve">C2-1404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-705</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-503</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-605</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1203A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-2003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1706</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1503</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-2006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1605</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1904</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-602</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1203A</t>
+    <t xml:space="preserve">c2-1402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-2004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-2006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B389</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1202A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c4-602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">480-481</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-1502</t>
   </si>
   <si>
     <t xml:space="preserve">c2-1702</t>
   </si>
   <si>
-    <t xml:space="preserve">C3-404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-803</t>
+    <t xml:space="preserve">C2-1802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-306</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-1805</t>
   </si>
   <si>
     <t xml:space="preserve">c1-804</t>
   </si>
   <si>
-    <t xml:space="preserve">C1-1705</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1204A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c4-405</t>
+    <t xml:space="preserve">C3-1703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-1905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c3-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5-1104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-1603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-1505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c2-1204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B375</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">490-491</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">551A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1105</t>
   </si>
   <si>
     <t xml:space="preserve">C1-1805</t>
   </si>
   <si>
-    <t xml:space="preserve">C2-1406</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c4-804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-1506</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c3-403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-1002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-2001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1706</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-2006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-306</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-1502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1203A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-405</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-1505</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c4-806</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1205A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1202A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c4-602</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1204A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1405</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1904</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1602</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-705</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c4-102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c3-1003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-1002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-1802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-2004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-1805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-405</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-406</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-506</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-1104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-2002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-406</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1745A</t>
+    <t xml:space="preserve">C4-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1972A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">424-425</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">525-526</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1914A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">540-541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B390</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B391</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B490</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B492</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-2005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1606</t>
   </si>
   <si>
     <t xml:space="preserve">C2-404</t>
@@ -7006,7 +7285,76 @@
     <t xml:space="preserve">C2-302</t>
   </si>
   <si>
-    <t xml:space="preserve">C1-2005</t>
+    <t xml:space="preserve">C1-601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B369</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-1704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B481</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-2005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B372</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2-1602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B371C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">455-456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-1601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B491</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B371B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B478</t>
   </si>
   <si>
     <t xml:space="preserve">C1-805</t>
@@ -7015,307 +7363,16 @@
     <t xml:space="preserve">C1-1201</t>
   </si>
   <si>
-    <t xml:space="preserve">C1-501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1914A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1972A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-405</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-706</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1401</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1401</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1606</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-806</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-605</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-505</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">424-425</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">426-427</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">428-429</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">430-431</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">439-440</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">442-443</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">445-446</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-2002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">448-449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">477A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2-902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">480-481</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">485-486</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">490-491</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-904</t>
-  </si>
-  <si>
-    <t xml:space="preserve">493-494</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">519-520</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">525-526</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">528-529</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">532-533</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c5-903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">532A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">536-537</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">538-539</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-503</t>
-  </si>
-  <si>
-    <t xml:space="preserve">540-541</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">547A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">551A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">557B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">558A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-606</t>
-  </si>
-  <si>
-    <t xml:space="preserve">565A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">583A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B361</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B369</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c1-301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B370B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B371B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-1602</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B371C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-2005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B372</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-606</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B375</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B389</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1-1804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B391</t>
+    <t xml:space="preserve">C3-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3-1802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B473</t>
   </si>
   <si>
     <t xml:space="preserve">C2-1405</t>
@@ -7324,46 +7381,19 @@
     <t xml:space="preserve">B472</t>
   </si>
   <si>
-    <t xml:space="preserve">C3-1802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B473</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B475</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B478</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2-806</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B479</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3-1204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B490</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4-1601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B491</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5-1902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B492</t>
+    <t xml:space="preserve">C4-604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B492A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5-401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B488</t>
   </si>
 </sst>
 </file>
@@ -7641,7 +7671,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B2133"/>
+  <dimension ref="A1:B2141"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22473,7 +22503,7 @@
         <v>2119</v>
       </c>
       <c r="B1854" s="2" t="n">
-        <v>433</v>
+        <v>463</v>
       </c>
     </row>
     <row r="1855" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22481,7 +22511,7 @@
         <v>2120</v>
       </c>
       <c r="B1855" s="2" t="n">
-        <v>434</v>
+        <v>441</v>
       </c>
     </row>
     <row r="1856" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22489,7 +22519,7 @@
         <v>2121</v>
       </c>
       <c r="B1856" s="2" t="n">
-        <v>441</v>
+        <v>462</v>
       </c>
     </row>
     <row r="1857" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22497,7 +22527,7 @@
         <v>2122</v>
       </c>
       <c r="B1857" s="2" t="n">
-        <v>452</v>
+        <v>459</v>
       </c>
     </row>
     <row r="1858" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22505,2207 +22535,2271 @@
         <v>2123</v>
       </c>
       <c r="B1858" s="2" t="n">
-        <v>453</v>
+        <v>465</v>
       </c>
     </row>
     <row r="1859" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1859" s="2" t="s">
         <v>2124</v>
       </c>
-      <c r="B1859" s="2" t="n">
-        <v>454</v>
+      <c r="B1859" s="2" t="s">
+        <v>2125</v>
       </c>
     </row>
     <row r="1860" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1860" s="2" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="B1860" s="2" t="n">
-        <v>459</v>
+        <v>473</v>
       </c>
     </row>
     <row r="1861" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1861" s="2" t="s">
-        <v>2126</v>
+        <v>2127</v>
       </c>
       <c r="B1861" s="2" t="n">
-        <v>462</v>
+        <v>474</v>
       </c>
     </row>
     <row r="1862" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1862" s="2" t="s">
-        <v>2127</v>
+        <v>2128</v>
       </c>
       <c r="B1862" s="2" t="n">
-        <v>463</v>
+        <v>546</v>
       </c>
     </row>
     <row r="1863" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1863" s="2" t="s">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="B1863" s="2" t="n">
-        <v>465</v>
+        <v>477</v>
       </c>
     </row>
     <row r="1864" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1864" s="2" t="s">
-        <v>2129</v>
+        <v>2130</v>
       </c>
       <c r="B1864" s="2" t="n">
-        <v>469</v>
+        <v>514</v>
       </c>
     </row>
     <row r="1865" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1865" s="2" t="s">
-        <v>2130</v>
+        <v>2131</v>
       </c>
       <c r="B1865" s="2" t="n">
-        <v>470</v>
+        <v>566</v>
       </c>
     </row>
     <row r="1866" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1866" s="2" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="B1866" s="2" t="n">
-        <v>471</v>
+        <v>563</v>
       </c>
     </row>
     <row r="1867" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1867" s="2" t="s">
-        <v>2132</v>
+        <v>2133</v>
       </c>
       <c r="B1867" s="2" t="n">
-        <v>472</v>
+        <v>567</v>
       </c>
     </row>
     <row r="1868" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1868" s="2" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="B1868" s="2" t="n">
-        <v>473</v>
+        <v>479</v>
       </c>
     </row>
     <row r="1869" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1869" s="2" t="s">
-        <v>2134</v>
+        <v>2135</v>
       </c>
       <c r="B1869" s="2" t="n">
-        <v>474</v>
+        <v>571</v>
       </c>
     </row>
     <row r="1870" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1870" s="2" t="s">
-        <v>2135</v>
+        <v>2136</v>
       </c>
       <c r="B1870" s="2" t="n">
-        <v>477</v>
+        <v>573</v>
       </c>
     </row>
     <row r="1871" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1871" s="2" t="s">
-        <v>2136</v>
+        <v>2137</v>
       </c>
       <c r="B1871" s="2" t="n">
-        <v>478</v>
+        <v>482</v>
       </c>
     </row>
     <row r="1872" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1872" s="2" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="B1872" s="2" t="n">
-        <v>479</v>
+        <v>555</v>
       </c>
     </row>
     <row r="1873" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1873" s="2" t="s">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="B1873" s="2" t="n">
-        <v>482</v>
+        <v>561</v>
       </c>
     </row>
     <row r="1874" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1874" s="2" t="s">
-        <v>2139</v>
-      </c>
-      <c r="B1874" s="2" t="n">
-        <v>484</v>
+        <v>2140</v>
+      </c>
+      <c r="B1874" s="2" t="s">
+        <v>2141</v>
       </c>
     </row>
     <row r="1875" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1875" s="2" t="s">
-        <v>2140</v>
+        <v>2142</v>
       </c>
       <c r="B1875" s="2" t="n">
-        <v>487</v>
+        <v>554</v>
       </c>
     </row>
     <row r="1876" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1876" s="2" t="s">
-        <v>2141</v>
+        <v>2143</v>
       </c>
       <c r="B1876" s="2" t="n">
-        <v>488</v>
+        <v>523</v>
       </c>
     </row>
     <row r="1877" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1877" s="2" t="s">
-        <v>2142</v>
-      </c>
-      <c r="B1877" s="2" t="n">
-        <v>489</v>
+        <v>2144</v>
+      </c>
+      <c r="B1877" s="2" t="s">
+        <v>2145</v>
       </c>
     </row>
     <row r="1878" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1878" s="2" t="s">
-        <v>2143</v>
+        <v>2146</v>
       </c>
       <c r="B1878" s="2" t="n">
-        <v>492</v>
+        <v>521</v>
       </c>
     </row>
     <row r="1879" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1879" s="2" t="s">
-        <v>2144</v>
+        <v>2147</v>
       </c>
       <c r="B1879" s="2" t="n">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="1880" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1880" s="2" t="s">
-        <v>2145</v>
+        <v>2148</v>
       </c>
       <c r="B1880" s="2" t="n">
-        <v>497</v>
+        <v>550</v>
       </c>
     </row>
     <row r="1881" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1881" s="2" t="s">
-        <v>2146</v>
+        <v>2149</v>
       </c>
       <c r="B1881" s="2" t="n">
-        <v>498</v>
+        <v>472</v>
       </c>
     </row>
     <row r="1882" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1882" s="2" t="s">
-        <v>2147</v>
+        <v>2150</v>
       </c>
       <c r="B1882" s="2" t="n">
-        <v>499</v>
+        <v>470</v>
       </c>
     </row>
     <row r="1883" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1883" s="2" t="s">
-        <v>2148</v>
+        <v>2151</v>
       </c>
       <c r="B1883" s="2" t="n">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="1884" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1884" s="2" t="s">
-        <v>2149</v>
+        <v>2152</v>
       </c>
       <c r="B1884" s="2" t="n">
-        <v>501</v>
+        <v>570</v>
       </c>
     </row>
     <row r="1885" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1885" s="2" t="s">
-        <v>2150</v>
+        <v>2153</v>
       </c>
       <c r="B1885" s="2" t="n">
-        <v>502</v>
+        <v>527</v>
       </c>
     </row>
     <row r="1886" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1886" s="2" t="s">
-        <v>2151</v>
+        <v>2154</v>
       </c>
       <c r="B1886" s="2" t="n">
-        <v>503</v>
+        <v>569</v>
       </c>
     </row>
     <row r="1887" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1887" s="2" t="s">
-        <v>2152</v>
+        <v>2155</v>
       </c>
       <c r="B1887" s="2" t="n">
-        <v>504</v>
+        <v>454</v>
       </c>
     </row>
     <row r="1888" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1888" s="2" t="s">
-        <v>2153</v>
-      </c>
-      <c r="B1888" s="2" t="n">
-        <v>505</v>
+        <v>2156</v>
+      </c>
+      <c r="B1888" s="2" t="s">
+        <v>2157</v>
       </c>
     </row>
     <row r="1889" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1889" s="2" t="s">
-        <v>2154</v>
+        <v>2158</v>
       </c>
       <c r="B1889" s="2" t="n">
-        <v>506</v>
+        <v>499</v>
       </c>
     </row>
     <row r="1890" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1890" s="2" t="s">
-        <v>2155</v>
+        <v>2159</v>
       </c>
       <c r="B1890" s="2" t="n">
-        <v>508</v>
+        <v>469</v>
       </c>
     </row>
     <row r="1891" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1891" s="2" t="s">
-        <v>2156</v>
+        <v>2160</v>
       </c>
       <c r="B1891" s="2" t="n">
-        <v>514</v>
+        <v>575</v>
       </c>
     </row>
     <row r="1892" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1892" s="2" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
       <c r="B1892" s="2" t="n">
-        <v>517</v>
+        <v>556</v>
       </c>
     </row>
     <row r="1893" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1893" s="2" t="s">
-        <v>2158</v>
+        <v>2162</v>
       </c>
       <c r="B1893" s="2" t="n">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="1894" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1894" s="2" t="s">
-        <v>2159</v>
+        <v>2163</v>
       </c>
       <c r="B1894" s="2" t="n">
-        <v>521</v>
+        <v>551</v>
       </c>
     </row>
     <row r="1895" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1895" s="2" t="s">
-        <v>2160</v>
+        <v>2164</v>
       </c>
       <c r="B1895" s="2" t="n">
-        <v>523</v>
+        <v>568</v>
       </c>
     </row>
     <row r="1896" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1896" s="2" t="s">
-        <v>2161</v>
+        <v>2165</v>
       </c>
       <c r="B1896" s="2" t="n">
-        <v>527</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="1897" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1897" s="2" t="s">
-        <v>2162</v>
-      </c>
-      <c r="B1897" s="2" t="n">
-        <v>535</v>
+        <v>2166</v>
+      </c>
+      <c r="B1897" s="2" t="s">
+        <v>2167</v>
       </c>
     </row>
     <row r="1898" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1898" s="2" t="s">
-        <v>2163</v>
-      </c>
-      <c r="B1898" s="2" t="n">
-        <v>540</v>
+        <v>2168</v>
+      </c>
+      <c r="B1898" s="2" t="s">
+        <v>2169</v>
       </c>
     </row>
     <row r="1899" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1899" s="2" t="s">
-        <v>2164</v>
+        <v>2170</v>
       </c>
       <c r="B1899" s="2" t="n">
-        <v>542</v>
+        <v>503</v>
       </c>
     </row>
     <row r="1900" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1900" s="2" t="s">
-        <v>2165</v>
+        <v>2171</v>
       </c>
       <c r="B1900" s="2" t="n">
-        <v>546</v>
+        <v>558</v>
       </c>
     </row>
     <row r="1901" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1901" s="2" t="s">
-        <v>2166</v>
+        <v>2172</v>
       </c>
       <c r="B1901" s="2" t="n">
-        <v>547</v>
+        <v>506</v>
       </c>
     </row>
     <row r="1902" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1902" s="2" t="s">
-        <v>2167</v>
+        <v>2173</v>
       </c>
       <c r="B1902" s="2" t="n">
-        <v>548</v>
+        <v>576</v>
       </c>
     </row>
     <row r="1903" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1903" s="2" t="s">
-        <v>2168</v>
+        <v>2174</v>
       </c>
       <c r="B1903" s="2" t="n">
-        <v>549</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="1904" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1904" s="2" t="s">
-        <v>2169</v>
+        <v>2175</v>
       </c>
       <c r="B1904" s="2" t="n">
-        <v>550</v>
+        <v>553</v>
       </c>
     </row>
     <row r="1905" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1905" s="2" t="s">
-        <v>2170</v>
+        <v>2176</v>
       </c>
       <c r="B1905" s="2" t="n">
-        <v>551</v>
+        <v>1912</v>
       </c>
     </row>
     <row r="1906" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1906" s="2" t="s">
-        <v>2171</v>
+        <v>2177</v>
       </c>
       <c r="B1906" s="2" t="n">
-        <v>552</v>
+        <v>505</v>
       </c>
     </row>
     <row r="1907" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1907" s="2" t="s">
-        <v>2172</v>
+        <v>2178</v>
       </c>
       <c r="B1907" s="2" t="n">
-        <v>553</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="1908" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1908" s="2" t="s">
-        <v>2173</v>
+        <v>2179</v>
       </c>
       <c r="B1908" s="2" t="n">
-        <v>554</v>
+        <v>535</v>
       </c>
     </row>
     <row r="1909" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1909" s="2" t="s">
-        <v>2174</v>
+        <v>2180</v>
       </c>
       <c r="B1909" s="2" t="n">
-        <v>555</v>
+        <v>504</v>
       </c>
     </row>
     <row r="1910" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1910" s="2" t="s">
-        <v>2175</v>
+        <v>2181</v>
       </c>
       <c r="B1910" s="2" t="n">
-        <v>556</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1911" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1911" s="2" t="s">
-        <v>2176</v>
+        <v>2182</v>
       </c>
       <c r="B1911" s="2" t="n">
-        <v>557</v>
+        <v>471</v>
       </c>
     </row>
     <row r="1912" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1912" s="2" t="s">
-        <v>2177</v>
+        <v>2183</v>
       </c>
       <c r="B1912" s="2" t="n">
-        <v>558</v>
+        <v>564</v>
       </c>
     </row>
     <row r="1913" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1913" s="2" t="s">
-        <v>2178</v>
+        <v>2184</v>
       </c>
       <c r="B1913" s="2" t="n">
-        <v>559</v>
+        <v>565</v>
       </c>
     </row>
     <row r="1914" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1914" s="2" t="s">
-        <v>2179</v>
+        <v>2185</v>
       </c>
       <c r="B1914" s="2" t="n">
-        <v>560</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="1915" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1915" s="2" t="s">
-        <v>2180</v>
+        <v>2186</v>
       </c>
       <c r="B1915" s="2" t="n">
-        <v>561</v>
+        <v>495</v>
       </c>
     </row>
     <row r="1916" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1916" s="2" t="s">
-        <v>2181</v>
+        <v>2187</v>
       </c>
       <c r="B1916" s="2" t="n">
-        <v>562</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="1917" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1917" s="2" t="s">
-        <v>2182</v>
+        <v>2188</v>
       </c>
       <c r="B1917" s="2" t="n">
-        <v>563</v>
+        <v>581</v>
       </c>
     </row>
     <row r="1918" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1918" s="2" t="s">
-        <v>2183</v>
+        <v>2189</v>
       </c>
       <c r="B1918" s="2" t="n">
-        <v>564</v>
+        <v>580</v>
       </c>
     </row>
     <row r="1919" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1919" s="2" t="s">
-        <v>2184</v>
-      </c>
-      <c r="B1919" s="2" t="n">
-        <v>565</v>
+        <v>2190</v>
+      </c>
+      <c r="B1919" s="2" t="s">
+        <v>2191</v>
       </c>
     </row>
     <row r="1920" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1920" s="2" t="s">
-        <v>2185</v>
+        <v>2192</v>
       </c>
       <c r="B1920" s="2" t="n">
-        <v>566</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="1921" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1921" s="2" t="s">
-        <v>2186</v>
+        <v>2193</v>
       </c>
       <c r="B1921" s="2" t="n">
-        <v>567</v>
+        <v>501</v>
       </c>
     </row>
     <row r="1922" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1922" s="2" t="s">
-        <v>2187</v>
-      </c>
-      <c r="B1922" s="2" t="n">
-        <v>568</v>
+        <v>2194</v>
+      </c>
+      <c r="B1922" s="2" t="s">
+        <v>2195</v>
       </c>
     </row>
     <row r="1923" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1923" s="2" t="s">
-        <v>2188</v>
+        <v>2196</v>
       </c>
       <c r="B1923" s="2" t="n">
-        <v>569</v>
+        <v>434</v>
       </c>
     </row>
     <row r="1924" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1924" s="2" t="s">
-        <v>2189</v>
+        <v>2197</v>
       </c>
       <c r="B1924" s="2" t="n">
-        <v>570</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1925" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1925" s="2" t="s">
-        <v>2190</v>
-      </c>
-      <c r="B1925" s="2" t="n">
-        <v>571</v>
+        <v>2198</v>
+      </c>
+      <c r="B1925" s="2" t="s">
+        <v>2199</v>
       </c>
     </row>
     <row r="1926" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1926" s="2" t="s">
-        <v>2191</v>
+        <v>2200</v>
       </c>
       <c r="B1926" s="2" t="n">
-        <v>572</v>
+        <v>452</v>
       </c>
     </row>
     <row r="1927" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1927" s="2" t="s">
-        <v>2192</v>
-      </c>
-      <c r="B1927" s="2" t="n">
-        <v>573</v>
+        <v>2201</v>
+      </c>
+      <c r="B1927" s="2" t="s">
+        <v>2202</v>
       </c>
     </row>
     <row r="1928" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1928" s="2" t="s">
-        <v>2193</v>
+        <v>2203</v>
       </c>
       <c r="B1928" s="2" t="n">
-        <v>574</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="1929" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1929" s="2" t="s">
-        <v>2194</v>
+        <v>2204</v>
       </c>
       <c r="B1929" s="2" t="n">
-        <v>575</v>
+        <v>584</v>
       </c>
     </row>
     <row r="1930" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1930" s="2" t="s">
-        <v>2195</v>
+        <v>2205</v>
       </c>
       <c r="B1930" s="2" t="n">
-        <v>576</v>
+        <v>559</v>
       </c>
     </row>
     <row r="1931" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1931" s="2" t="s">
-        <v>2196</v>
-      </c>
-      <c r="B1931" s="2" t="n">
-        <v>577</v>
+        <v>2206</v>
+      </c>
+      <c r="B1931" s="2" t="s">
+        <v>2207</v>
       </c>
     </row>
     <row r="1932" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1932" s="2" t="s">
-        <v>2197</v>
+        <v>2208</v>
       </c>
       <c r="B1932" s="2" t="n">
-        <v>578</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="1933" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1933" s="2" t="s">
-        <v>2198</v>
+        <v>2209</v>
       </c>
       <c r="B1933" s="2" t="n">
-        <v>579</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="1934" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1934" s="2" t="s">
-        <v>2199</v>
-      </c>
-      <c r="B1934" s="2" t="n">
-        <v>580</v>
+        <v>2210</v>
+      </c>
+      <c r="B1934" s="2" t="s">
+        <v>2211</v>
       </c>
     </row>
     <row r="1935" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1935" s="2" t="s">
-        <v>2200</v>
-      </c>
-      <c r="B1935" s="2" t="n">
-        <v>581</v>
+        <v>2212</v>
+      </c>
+      <c r="B1935" s="2" t="s">
+        <v>2213</v>
       </c>
     </row>
     <row r="1936" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1936" s="2" t="s">
-        <v>2201</v>
+        <v>2214</v>
       </c>
       <c r="B1936" s="2" t="n">
-        <v>582</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="1937" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1937" s="2" t="s">
-        <v>2202</v>
-      </c>
-      <c r="B1937" s="2" t="n">
-        <v>583</v>
+        <v>2215</v>
+      </c>
+      <c r="B1937" s="2" t="s">
+        <v>1658</v>
       </c>
     </row>
     <row r="1938" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1938" s="2" t="s">
-        <v>2203</v>
+        <v>2216</v>
       </c>
       <c r="B1938" s="2" t="n">
-        <v>584</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1939" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1939" s="2" t="s">
-        <v>2204</v>
+        <v>2217</v>
       </c>
       <c r="B1939" s="2" t="n">
-        <v>585</v>
+        <v>500</v>
       </c>
     </row>
     <row r="1940" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1940" s="2" t="s">
-        <v>2205</v>
+        <v>2218</v>
       </c>
       <c r="B1940" s="2" t="n">
-        <v>586</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="1941" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1941" s="2" t="s">
-        <v>2206</v>
-      </c>
-      <c r="B1941" s="2" t="n">
-        <v>588</v>
+        <v>2219</v>
+      </c>
+      <c r="B1941" s="2" t="s">
+        <v>1658</v>
       </c>
     </row>
     <row r="1942" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1942" s="2" t="s">
-        <v>2207</v>
+        <v>2220</v>
       </c>
       <c r="B1942" s="2" t="n">
-        <v>1745</v>
+        <v>492</v>
       </c>
     </row>
     <row r="1943" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1943" s="2" t="s">
-        <v>2208</v>
-      </c>
-      <c r="B1943" s="2" t="n">
-        <v>1792</v>
+        <v>2221</v>
+      </c>
+      <c r="B1943" s="2" t="s">
+        <v>2222</v>
       </c>
     </row>
     <row r="1944" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1944" s="2" t="s">
-        <v>2209</v>
+        <v>2223</v>
       </c>
       <c r="B1944" s="2" t="n">
-        <v>1793</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="1945" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1945" s="2" t="s">
-        <v>2210</v>
+        <v>2224</v>
       </c>
       <c r="B1945" s="2" t="n">
-        <v>1796</v>
+        <v>562</v>
       </c>
     </row>
     <row r="1946" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1946" s="2" t="s">
-        <v>2211</v>
+        <v>2225</v>
       </c>
       <c r="B1946" s="2" t="n">
-        <v>1850</v>
+        <v>508</v>
       </c>
     </row>
     <row r="1947" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1947" s="2" t="s">
-        <v>2212</v>
+        <v>2226</v>
       </c>
       <c r="B1947" s="2" t="n">
-        <v>1851</v>
+        <v>517</v>
       </c>
     </row>
     <row r="1948" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1948" s="2" t="s">
-        <v>2213</v>
+        <v>2227</v>
       </c>
       <c r="B1948" s="2" t="n">
-        <v>1853</v>
+        <v>498</v>
       </c>
     </row>
     <row r="1949" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1949" s="2" t="s">
-        <v>2214</v>
+        <v>2228</v>
       </c>
       <c r="B1949" s="2" t="n">
-        <v>1855</v>
+        <v>560</v>
       </c>
     </row>
     <row r="1950" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1950" s="2" t="s">
-        <v>2215</v>
+        <v>2229</v>
       </c>
       <c r="B1950" s="2" t="n">
-        <v>1856</v>
+        <v>557</v>
       </c>
     </row>
     <row r="1951" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1951" s="2" t="s">
-        <v>2216</v>
-      </c>
-      <c r="B1951" s="2" t="n">
-        <v>1857</v>
+        <v>2230</v>
+      </c>
+      <c r="B1951" s="2" t="s">
+        <v>2231</v>
       </c>
     </row>
     <row r="1952" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1952" s="2" t="s">
-        <v>2217</v>
+        <v>2232</v>
       </c>
       <c r="B1952" s="2" t="n">
-        <v>1858</v>
+        <v>548</v>
       </c>
     </row>
     <row r="1953" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1953" s="2" t="s">
-        <v>2218</v>
+        <v>2233</v>
       </c>
       <c r="B1953" s="2" t="n">
-        <v>1898</v>
+        <v>487</v>
       </c>
     </row>
     <row r="1954" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1954" s="2" t="s">
-        <v>2219</v>
+        <v>2234</v>
       </c>
       <c r="B1954" s="2" t="n">
-        <v>1905</v>
+        <v>518</v>
       </c>
     </row>
     <row r="1955" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1955" s="2" t="s">
-        <v>2220</v>
+        <v>2235</v>
       </c>
       <c r="B1955" s="2" t="n">
-        <v>1907</v>
+        <v>578</v>
       </c>
     </row>
     <row r="1956" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1956" s="2" t="s">
-        <v>2221</v>
+        <v>2236</v>
       </c>
       <c r="B1956" s="2" t="n">
-        <v>1908</v>
+        <v>579</v>
       </c>
     </row>
     <row r="1957" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1957" s="2" t="s">
-        <v>2222</v>
+        <v>2237</v>
       </c>
       <c r="B1957" s="2" t="n">
-        <v>1910</v>
+        <v>502</v>
       </c>
     </row>
     <row r="1958" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1958" s="2" t="s">
-        <v>2223</v>
-      </c>
-      <c r="B1958" s="2" t="n">
-        <v>1911</v>
+        <v>2238</v>
+      </c>
+      <c r="B1958" s="2" t="s">
+        <v>2239</v>
       </c>
     </row>
     <row r="1959" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1959" s="2" t="s">
-        <v>2224</v>
+        <v>2240</v>
       </c>
       <c r="B1959" s="2" t="n">
-        <v>1912</v>
+        <v>583</v>
       </c>
     </row>
     <row r="1960" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1960" s="2" t="s">
-        <v>2225</v>
+        <v>2241</v>
       </c>
       <c r="B1960" s="2" t="n">
-        <v>1913</v>
+        <v>577</v>
       </c>
     </row>
     <row r="1961" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1961" s="2" t="s">
-        <v>2226</v>
-      </c>
-      <c r="B1961" s="2" t="n">
-        <v>1914</v>
+        <v>2242</v>
+      </c>
+      <c r="B1961" s="2" t="s">
+        <v>2243</v>
       </c>
     </row>
     <row r="1962" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1962" s="2" t="s">
-        <v>2227</v>
+        <v>2244</v>
       </c>
       <c r="B1962" s="2" t="n">
-        <v>1915</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="1963" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1963" s="2" t="s">
-        <v>2228</v>
+        <v>2245</v>
       </c>
       <c r="B1963" s="2" t="n">
-        <v>1916</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="1964" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1964" s="2" t="s">
-        <v>2229</v>
+        <v>2246</v>
       </c>
       <c r="B1964" s="2" t="n">
-        <v>1917</v>
+        <v>478</v>
       </c>
     </row>
     <row r="1965" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1965" s="2" t="s">
-        <v>2230</v>
+        <v>2247</v>
       </c>
       <c r="B1965" s="2" t="n">
-        <v>1918</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="1966" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1966" s="2" t="s">
-        <v>2231</v>
+        <v>2248</v>
       </c>
       <c r="B1966" s="2" t="n">
-        <v>1919</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="1967" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1967" s="2" t="s">
-        <v>2232</v>
+        <v>2249</v>
       </c>
       <c r="B1967" s="2" t="n">
-        <v>1920</v>
+        <v>574</v>
       </c>
     </row>
     <row r="1968" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1968" s="2" t="s">
-        <v>2233</v>
+        <v>2250</v>
       </c>
       <c r="B1968" s="2" t="n">
-        <v>1921</v>
+        <v>549</v>
       </c>
     </row>
     <row r="1969" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1969" s="2" t="s">
-        <v>2234</v>
+        <v>2251</v>
       </c>
       <c r="B1969" s="2" t="n">
-        <v>1922</v>
+        <v>572</v>
       </c>
     </row>
     <row r="1970" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1970" s="2" t="s">
-        <v>2235</v>
+        <v>2252</v>
       </c>
       <c r="B1970" s="2" t="n">
-        <v>1923</v>
+        <v>453</v>
       </c>
     </row>
     <row r="1971" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1971" s="2" t="s">
-        <v>2236</v>
+        <v>2253</v>
       </c>
       <c r="B1971" s="2" t="n">
-        <v>1925</v>
+        <v>582</v>
       </c>
     </row>
     <row r="1972" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1972" s="2" t="s">
-        <v>2237</v>
+        <v>2254</v>
       </c>
       <c r="B1972" s="2" t="n">
-        <v>1960</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="1973" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1973" s="2" t="s">
-        <v>2238</v>
+        <v>2255</v>
       </c>
       <c r="B1973" s="2" t="n">
-        <v>1961</v>
+        <v>2095</v>
       </c>
     </row>
     <row r="1974" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1974" s="2" t="s">
-        <v>2239</v>
-      </c>
-      <c r="B1974" s="2" t="n">
-        <v>1962</v>
+        <v>2256</v>
+      </c>
+      <c r="B1974" s="2" t="s">
+        <v>2257</v>
       </c>
     </row>
     <row r="1975" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1975" s="2" t="s">
-        <v>2240</v>
+        <v>2258</v>
       </c>
       <c r="B1975" s="2" t="n">
-        <v>1963</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="1976" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1976" s="2" t="s">
-        <v>2241</v>
+        <v>2259</v>
       </c>
       <c r="B1976" s="2" t="n">
-        <v>1964</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="1977" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1977" s="2" t="s">
-        <v>2242</v>
+        <v>2260</v>
       </c>
       <c r="B1977" s="2" t="n">
-        <v>1966</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="1978" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1978" s="2" t="s">
-        <v>2243</v>
+        <v>2261</v>
       </c>
       <c r="B1978" s="2" t="n">
-        <v>1967</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="1979" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1979" s="2" t="s">
-        <v>2244</v>
+        <v>2262</v>
       </c>
       <c r="B1979" s="2" t="n">
-        <v>1968</v>
+        <v>489</v>
       </c>
     </row>
     <row r="1980" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1980" s="2" t="s">
-        <v>2245</v>
+        <v>2263</v>
       </c>
       <c r="B1980" s="2" t="n">
-        <v>1971</v>
+        <v>588</v>
       </c>
     </row>
     <row r="1981" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1981" s="2" t="s">
-        <v>2246</v>
-      </c>
-      <c r="B1981" s="2" t="n">
-        <v>1972</v>
+        <v>2264</v>
+      </c>
+      <c r="B1981" s="2" t="s">
+        <v>2265</v>
       </c>
     </row>
     <row r="1982" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1982" s="2" t="s">
-        <v>2247</v>
+        <v>2266</v>
       </c>
       <c r="B1982" s="2" t="n">
-        <v>1973</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="1983" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1983" s="2" t="s">
-        <v>2248</v>
+        <v>2267</v>
       </c>
       <c r="B1983" s="2" t="n">
-        <v>1974</v>
+        <v>552</v>
       </c>
     </row>
     <row r="1984" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1984" s="2" t="s">
-        <v>2249</v>
-      </c>
-      <c r="B1984" s="2" t="n">
-        <v>1975</v>
+        <v>2268</v>
+      </c>
+      <c r="B1984" s="2" t="s">
+        <v>2269</v>
       </c>
     </row>
     <row r="1985" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1985" s="2" t="s">
-        <v>2250</v>
+        <v>2270</v>
       </c>
       <c r="B1985" s="2" t="n">
-        <v>1976</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="1986" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1986" s="2" t="s">
-        <v>2251</v>
+        <v>2271</v>
       </c>
       <c r="B1986" s="2" t="n">
-        <v>1977</v>
+        <v>1922</v>
       </c>
     </row>
     <row r="1987" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1987" s="2" t="s">
-        <v>2252</v>
+        <v>2272</v>
       </c>
       <c r="B1987" s="2" t="n">
-        <v>1978</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="1988" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1988" s="2" t="s">
-        <v>2253</v>
+        <v>2273</v>
       </c>
       <c r="B1988" s="2" t="n">
-        <v>2014</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="1989" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1989" s="2" t="s">
-        <v>2254</v>
+        <v>2274</v>
       </c>
       <c r="B1989" s="2" t="n">
-        <v>2015</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="1990" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1990" s="2" t="s">
-        <v>2255</v>
+        <v>2275</v>
       </c>
       <c r="B1990" s="2" t="n">
-        <v>2016</v>
+        <v>1918</v>
       </c>
     </row>
     <row r="1991" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1991" s="2" t="s">
-        <v>2256</v>
+        <v>2276</v>
       </c>
       <c r="B1991" s="2" t="n">
-        <v>2017</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="1992" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1992" s="2" t="s">
-        <v>2257</v>
+        <v>2277</v>
       </c>
       <c r="B1992" s="2" t="n">
-        <v>2018</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="1993" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1993" s="2" t="s">
-        <v>2258</v>
+        <v>2278</v>
       </c>
       <c r="B1993" s="2" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="1994" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1994" s="2" t="s">
-        <v>2259</v>
+        <v>2279</v>
       </c>
       <c r="B1994" s="2" t="n">
-        <v>2020</v>
+        <v>540</v>
       </c>
     </row>
     <row r="1995" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1995" s="2" t="s">
-        <v>2260</v>
+        <v>2280</v>
       </c>
       <c r="B1995" s="2" t="n">
-        <v>2021</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="1996" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1996" s="2" t="s">
-        <v>2261</v>
+        <v>2281</v>
       </c>
       <c r="B1996" s="2" t="n">
-        <v>2022</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="1997" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1997" s="2" t="s">
-        <v>2262</v>
+        <v>2282</v>
       </c>
       <c r="B1997" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="1998" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1998" s="2" t="s">
-        <v>2263</v>
+        <v>2283</v>
       </c>
       <c r="B1998" s="2" t="n">
-        <v>2027</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="1999" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1999" s="2" t="s">
-        <v>2264</v>
+        <v>2284</v>
       </c>
       <c r="B1999" s="2" t="n">
-        <v>2028</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="2000" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2000" s="2" t="s">
-        <v>2265</v>
-      </c>
-      <c r="B2000" s="2" t="n">
-        <v>2029</v>
+        <v>2285</v>
+      </c>
+      <c r="B2000" s="2" t="s">
+        <v>2286</v>
       </c>
     </row>
     <row r="2001" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2001" s="2" t="s">
-        <v>2266</v>
-      </c>
-      <c r="B2001" s="2" t="n">
-        <v>2030</v>
+        <v>2287</v>
+      </c>
+      <c r="B2001" s="2" t="s">
+        <v>2288</v>
       </c>
     </row>
     <row r="2002" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2002" s="2" t="s">
-        <v>2267</v>
+        <v>2289</v>
       </c>
       <c r="B2002" s="2" t="n">
-        <v>2031</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="2003" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2003" s="2" t="s">
-        <v>2268</v>
+        <v>2290</v>
       </c>
       <c r="B2003" s="2" t="n">
-        <v>2032</v>
+        <v>2190</v>
       </c>
     </row>
     <row r="2004" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2004" s="2" t="s">
-        <v>2269</v>
+        <v>2291</v>
       </c>
       <c r="B2004" s="2" t="n">
-        <v>2033</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="2005" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2005" s="2" t="s">
-        <v>2270</v>
+        <v>2292</v>
       </c>
       <c r="B2005" s="2" t="n">
-        <v>2034</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="2006" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2006" s="2" t="s">
-        <v>2271</v>
-      </c>
-      <c r="B2006" s="2" t="n">
-        <v>2035</v>
+        <v>2293</v>
+      </c>
+      <c r="B2006" s="2" t="s">
+        <v>2294</v>
       </c>
     </row>
     <row r="2007" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2007" s="2" t="s">
-        <v>2272</v>
+        <v>2295</v>
       </c>
       <c r="B2007" s="2" t="n">
-        <v>2088</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="2008" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2008" s="2" t="s">
-        <v>2273</v>
+        <v>2296</v>
       </c>
       <c r="B2008" s="2" t="n">
-        <v>2090</v>
+        <v>542</v>
       </c>
     </row>
     <row r="2009" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2009" s="2" t="s">
-        <v>2274</v>
+        <v>2297</v>
       </c>
       <c r="B2009" s="2" t="n">
-        <v>2091</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="2010" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2010" s="2" t="s">
-        <v>2275</v>
+        <v>2298</v>
       </c>
       <c r="B2010" s="2" t="n">
-        <v>2092</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="2011" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2011" s="2" t="s">
-        <v>2276</v>
+        <v>2299</v>
       </c>
       <c r="B2011" s="2" t="n">
-        <v>2093</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="2012" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2012" s="2" t="s">
-        <v>2277</v>
+        <v>2300</v>
       </c>
       <c r="B2012" s="2" t="n">
-        <v>2094</v>
+        <v>2184</v>
       </c>
     </row>
     <row r="2013" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2013" s="2" t="s">
-        <v>2278</v>
+        <v>2301</v>
       </c>
       <c r="B2013" s="2" t="n">
-        <v>2095</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="2014" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2014" s="2" t="s">
-        <v>2279</v>
-      </c>
-      <c r="B2014" s="2" t="n">
-        <v>2096</v>
+        <v>2302</v>
+      </c>
+      <c r="B2014" s="2" t="s">
+        <v>2303</v>
       </c>
     </row>
     <row r="2015" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2015" s="2" t="s">
-        <v>2280</v>
+        <v>2304</v>
       </c>
       <c r="B2015" s="2" t="n">
-        <v>2097</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="2016" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2016" s="2" t="s">
-        <v>2281</v>
+        <v>2305</v>
       </c>
       <c r="B2016" s="2" t="n">
-        <v>2098</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="2017" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2017" s="2" t="s">
-        <v>2282</v>
+        <v>2306</v>
       </c>
       <c r="B2017" s="2" t="n">
-        <v>2099</v>
+        <v>2261</v>
       </c>
     </row>
     <row r="2018" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2018" s="2" t="s">
-        <v>2283</v>
+        <v>2307</v>
       </c>
       <c r="B2018" s="2" t="n">
-        <v>2102</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="2019" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2019" s="2" t="s">
-        <v>2284</v>
+        <v>2308</v>
       </c>
       <c r="B2019" s="2" t="n">
-        <v>2103</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="2020" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2020" s="2" t="s">
-        <v>2285</v>
+        <v>2309</v>
       </c>
       <c r="B2020" s="2" t="n">
-        <v>2104</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="2021" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2021" s="2" t="s">
-        <v>2286</v>
+        <v>2310</v>
       </c>
       <c r="B2021" s="2" t="n">
-        <v>2105</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="2022" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2022" s="2" t="s">
-        <v>2287</v>
+        <v>2311</v>
       </c>
       <c r="B2022" s="2" t="n">
-        <v>2106</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="2023" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2023" s="2" t="s">
-        <v>2288</v>
-      </c>
-      <c r="B2023" s="2" t="n">
-        <v>2107</v>
+        <v>2312</v>
+      </c>
+      <c r="B2023" s="2" t="s">
+        <v>2313</v>
       </c>
     </row>
     <row r="2024" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2024" s="2" t="s">
-        <v>2289</v>
+        <v>2314</v>
       </c>
       <c r="B2024" s="2" t="n">
-        <v>2109</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="2025" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2025" s="2" t="s">
-        <v>2290</v>
+        <v>2315</v>
       </c>
       <c r="B2025" s="2" t="n">
-        <v>2110</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="2026" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2026" s="2" t="s">
-        <v>2291</v>
+        <v>2316</v>
       </c>
       <c r="B2026" s="2" t="n">
-        <v>2112</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="2027" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2027" s="2" t="s">
-        <v>2292</v>
+        <v>2317</v>
       </c>
       <c r="B2027" s="2" t="n">
-        <v>2113</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="2028" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2028" s="2" t="s">
-        <v>2293</v>
+        <v>2318</v>
       </c>
       <c r="B2028" s="2" t="n">
-        <v>2114</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="2029" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2029" s="2" t="s">
-        <v>2294</v>
+        <v>2319</v>
       </c>
       <c r="B2029" s="2" t="n">
-        <v>2170</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="2030" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2030" s="2" t="s">
-        <v>2295</v>
+        <v>2320</v>
       </c>
       <c r="B2030" s="2" t="n">
-        <v>2171</v>
+        <v>586</v>
       </c>
     </row>
     <row r="2031" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2031" s="2" t="s">
-        <v>2296</v>
+        <v>2321</v>
       </c>
       <c r="B2031" s="2" t="n">
-        <v>2172</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="2032" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2032" s="2" t="s">
-        <v>2297</v>
+        <v>2322</v>
       </c>
       <c r="B2032" s="2" t="n">
-        <v>2173</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="2033" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2033" s="2" t="s">
-        <v>2298</v>
+        <v>2323</v>
       </c>
       <c r="B2033" s="2" t="n">
-        <v>2174</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="2034" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2034" s="2" t="s">
-        <v>2299</v>
+        <v>2324</v>
       </c>
       <c r="B2034" s="2" t="n">
-        <v>2176</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="2035" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2035" s="2" t="s">
-        <v>2300</v>
+        <v>2325</v>
       </c>
       <c r="B2035" s="2" t="n">
-        <v>2177</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="2036" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2036" s="2" t="s">
-        <v>2301</v>
+        <v>2326</v>
       </c>
       <c r="B2036" s="2" t="n">
-        <v>2178</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="2037" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2037" s="2" t="s">
-        <v>2302</v>
+        <v>2327</v>
       </c>
       <c r="B2037" s="2" t="n">
-        <v>2179</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="2038" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2038" s="2" t="s">
-        <v>2303</v>
+        <v>2328</v>
       </c>
       <c r="B2038" s="2" t="n">
-        <v>2180</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="2039" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2039" s="2" t="s">
-        <v>2304</v>
+        <v>2329</v>
       </c>
       <c r="B2039" s="2" t="n">
-        <v>2181</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="2040" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2040" s="2" t="s">
-        <v>2305</v>
+        <v>2330</v>
       </c>
       <c r="B2040" s="2" t="n">
-        <v>2183</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="2041" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2041" s="2" t="s">
-        <v>2306</v>
+        <v>2331</v>
       </c>
       <c r="B2041" s="2" t="n">
-        <v>2184</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="2042" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2042" s="2" t="s">
-        <v>2307</v>
+        <v>2332</v>
       </c>
       <c r="B2042" s="2" t="n">
-        <v>2185</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="2043" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2043" s="2" t="s">
-        <v>2308</v>
-      </c>
-      <c r="B2043" s="2" t="n">
-        <v>2186</v>
+        <v>2333</v>
+      </c>
+      <c r="B2043" s="2" t="s">
+        <v>2334</v>
       </c>
     </row>
     <row r="2044" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2044" s="2" t="s">
-        <v>2309</v>
+        <v>2335</v>
       </c>
       <c r="B2044" s="2" t="n">
-        <v>2187</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="2045" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2045" s="2" t="s">
-        <v>2310</v>
+        <v>2336</v>
       </c>
       <c r="B2045" s="2" t="n">
-        <v>2188</v>
+        <v>585</v>
       </c>
     </row>
     <row r="2046" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2046" s="2" t="s">
-        <v>2311</v>
+        <v>2337</v>
       </c>
       <c r="B2046" s="2" t="n">
-        <v>2189</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="2047" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2047" s="2" t="s">
-        <v>2312</v>
+        <v>2338</v>
       </c>
       <c r="B2047" s="2" t="n">
-        <v>2190</v>
+        <v>2264</v>
       </c>
     </row>
     <row r="2048" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2048" s="2" t="s">
-        <v>2313</v>
+        <v>2339</v>
       </c>
       <c r="B2048" s="2" t="n">
-        <v>2191</v>
+        <v>1964</v>
       </c>
     </row>
     <row r="2049" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2049" s="2" t="s">
-        <v>2314</v>
+        <v>2340</v>
       </c>
       <c r="B2049" s="2" t="n">
-        <v>2256</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="2050" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2050" s="2" t="s">
-        <v>2315</v>
+        <v>2341</v>
       </c>
       <c r="B2050" s="2" t="n">
-        <v>2257</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="2051" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2051" s="2" t="s">
-        <v>2316</v>
+        <v>2342</v>
       </c>
       <c r="B2051" s="2" t="n">
-        <v>2258</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="2052" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2052" s="2" t="s">
-        <v>2317</v>
+        <v>2343</v>
       </c>
       <c r="B2052" s="2" t="n">
-        <v>2259</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="2053" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2053" s="2" t="s">
-        <v>2318</v>
-      </c>
-      <c r="B2053" s="2" t="n">
-        <v>2260</v>
+        <v>2344</v>
+      </c>
+      <c r="B2053" s="2" t="s">
+        <v>1658</v>
       </c>
     </row>
     <row r="2054" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2054" s="2" t="s">
-        <v>2319</v>
+        <v>2345</v>
       </c>
       <c r="B2054" s="2" t="n">
-        <v>2261</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="2055" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2055" s="2" t="s">
-        <v>2320</v>
-      </c>
-      <c r="B2055" s="2" t="n">
-        <v>2262</v>
+        <v>2346</v>
+      </c>
+      <c r="B2055" s="2" t="s">
+        <v>1658</v>
       </c>
     </row>
     <row r="2056" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2056" s="2" t="s">
-        <v>2321</v>
+        <v>2347</v>
       </c>
       <c r="B2056" s="2" t="n">
-        <v>2263</v>
+        <v>2260</v>
       </c>
     </row>
     <row r="2057" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2057" s="2" t="s">
-        <v>2322</v>
+        <v>2348</v>
       </c>
       <c r="B2057" s="2" t="n">
-        <v>2264</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="2058" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2058" s="2" t="s">
-        <v>2323</v>
-      </c>
-      <c r="B2058" s="2" t="s">
-        <v>2324</v>
+        <v>2349</v>
+      </c>
+      <c r="B2058" s="2" t="n">
+        <v>2105</v>
       </c>
     </row>
     <row r="2059" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2059" s="2" t="s">
-        <v>2325</v>
+        <v>2350</v>
       </c>
       <c r="B2059" s="2" t="n">
-        <v>1859</v>
+        <v>2107</v>
       </c>
     </row>
     <row r="2060" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2060" s="2" t="s">
-        <v>2326</v>
+        <v>2351</v>
       </c>
       <c r="B2060" s="2" t="n">
-        <v>1860</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="2061" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2061" s="2" t="s">
-        <v>2327</v>
+        <v>2352</v>
       </c>
       <c r="B2061" s="2" t="n">
-        <v>1861</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="2062" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2062" s="2" t="s">
-        <v>2328</v>
+        <v>2353</v>
       </c>
       <c r="B2062" s="2" t="n">
-        <v>1863</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="2063" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2063" s="2" t="s">
-        <v>2329</v>
+        <v>2354</v>
       </c>
       <c r="B2063" s="2" t="n">
-        <v>1902</v>
+        <v>2180</v>
       </c>
     </row>
     <row r="2064" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2064" s="2" t="s">
-        <v>2330</v>
+        <v>2355</v>
       </c>
       <c r="B2064" s="2" t="n">
-        <v>1903</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="2065" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2065" s="2" t="s">
-        <v>2331</v>
+        <v>2356</v>
       </c>
       <c r="B2065" s="2" t="n">
-        <v>1904</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="2066" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2066" s="2" t="s">
-        <v>2332</v>
-      </c>
-      <c r="B2066" s="2" t="s">
-        <v>2333</v>
+        <v>2357</v>
+      </c>
+      <c r="B2066" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="2067" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2067" s="2" t="s">
-        <v>2334</v>
+        <v>2358</v>
       </c>
       <c r="B2067" s="2" t="n">
-        <v>1958</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="2068" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2068" s="2" t="s">
-        <v>2335</v>
+        <v>2359</v>
       </c>
       <c r="B2068" s="2" t="n">
-        <v>1959</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="2069" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2069" s="2" t="s">
-        <v>2336</v>
+        <v>2360</v>
       </c>
       <c r="B2069" s="2" t="n">
-        <v>1965</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="2070" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2070" s="2" t="s">
-        <v>2337</v>
-      </c>
-      <c r="B2070" s="2" t="s">
-        <v>2338</v>
+        <v>2361</v>
+      </c>
+      <c r="B2070" s="2" t="n">
+        <v>2094</v>
       </c>
     </row>
     <row r="2071" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2071" s="2" t="s">
-        <v>2339</v>
+        <v>2362</v>
       </c>
       <c r="B2071" s="2" t="n">
-        <v>1979</v>
+        <v>2258</v>
       </c>
     </row>
     <row r="2072" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2072" s="2" t="s">
-        <v>2340</v>
+        <v>2363</v>
       </c>
       <c r="B2072" s="2" t="n">
-        <v>1980</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="2073" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2073" s="2" t="s">
-        <v>2341</v>
+        <v>2364</v>
       </c>
       <c r="B2073" s="2" t="n">
-        <v>1981</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="2074" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2074" s="2" t="s">
-        <v>2342</v>
+        <v>2365</v>
       </c>
       <c r="B2074" s="2" t="n">
-        <v>2013</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="2075" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2075" s="2" t="s">
-        <v>2343</v>
-      </c>
-      <c r="B2075" s="2" t="s">
-        <v>2344</v>
+        <v>2366</v>
+      </c>
+      <c r="B2075" s="2" t="n">
+        <v>2257</v>
       </c>
     </row>
     <row r="2076" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2076" s="2" t="s">
-        <v>2345</v>
+        <v>2367</v>
       </c>
       <c r="B2076" s="2" t="n">
-        <v>2037</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="2077" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2077" s="2" t="s">
-        <v>2346</v>
+        <v>2368</v>
       </c>
       <c r="B2077" s="2" t="n">
-        <v>2038</v>
+        <v>1976</v>
       </c>
     </row>
     <row r="2078" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2078" s="2" t="s">
-        <v>2347</v>
+        <v>2369</v>
       </c>
       <c r="B2078" s="2" t="n">
-        <v>2039</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="2079" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2079" s="2" t="s">
-        <v>2348</v>
+        <v>2370</v>
       </c>
       <c r="B2079" s="2" t="n">
-        <v>2040</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="2080" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2080" s="2" t="s">
-        <v>2349</v>
+        <v>2371</v>
       </c>
       <c r="B2080" s="2" t="n">
-        <v>2089</v>
+        <v>2256</v>
       </c>
     </row>
     <row r="2081" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2081" s="2" t="s">
-        <v>2350</v>
+        <v>2372</v>
       </c>
       <c r="B2081" s="2" t="n">
-        <v>2108</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="2082" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2082" s="2" t="s">
-        <v>2351</v>
+        <v>2373</v>
       </c>
       <c r="B2082" s="2" t="n">
-        <v>2192</v>
+        <v>2033</v>
       </c>
     </row>
     <row r="2083" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2083" s="2" t="s">
-        <v>2352</v>
+        <v>2374</v>
       </c>
       <c r="B2083" s="2" t="n">
-        <v>2193</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="2084" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2084" s="2" t="s">
-        <v>2353</v>
+        <v>2375</v>
       </c>
       <c r="B2084" s="2" t="n">
-        <v>2194</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="2085" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2085" s="2" t="s">
-        <v>2354</v>
+        <v>2376</v>
       </c>
       <c r="B2085" s="2" t="n">
-        <v>2253</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="2086" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2086" s="2" t="s">
-        <v>2355</v>
+        <v>2377</v>
       </c>
       <c r="B2086" s="2" t="n">
-        <v>2254</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="2087" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2087" s="2" t="s">
-        <v>2356</v>
-      </c>
-      <c r="B2087" s="2" t="n">
-        <v>2255</v>
+        <v>2378</v>
+      </c>
+      <c r="B2087" s="2" t="s">
+        <v>2379</v>
       </c>
     </row>
     <row r="2088" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2088" s="2" t="s">
-        <v>2357</v>
-      </c>
-      <c r="B2088" s="2" t="s">
-        <v>2358</v>
+        <v>2380</v>
+      </c>
+      <c r="B2088" s="2" t="n">
+        <v>1978</v>
       </c>
     </row>
     <row r="2089" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2089" s="2" t="s">
-        <v>2359</v>
+        <v>2381</v>
       </c>
       <c r="B2089" s="2" t="s">
-        <v>2360</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="2090" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2090" s="2" t="s">
-        <v>2361</v>
+        <v>2383</v>
       </c>
       <c r="B2090" s="2" t="s">
-        <v>2362</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="2091" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2091" s="2" t="s">
-        <v>2363</v>
-      </c>
-      <c r="B2091" s="2" t="s">
-        <v>2364</v>
+        <v>2385</v>
+      </c>
+      <c r="B2091" s="2" t="n">
+        <v>2097</v>
       </c>
     </row>
     <row r="2092" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2092" s="2" t="s">
-        <v>2365</v>
-      </c>
-      <c r="B2092" s="2" t="s">
-        <v>2366</v>
+        <v>2386</v>
+      </c>
+      <c r="B2092" s="2" t="n">
+        <v>1916</v>
       </c>
     </row>
     <row r="2093" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2093" s="2" t="s">
-        <v>2367</v>
+        <v>2387</v>
       </c>
       <c r="B2093" s="2" t="s">
-        <v>2368</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="2094" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2094" s="2" t="s">
-        <v>2369</v>
+        <v>2389</v>
       </c>
       <c r="B2094" s="2" t="s">
-        <v>2370</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="2095" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2095" s="2" t="s">
-        <v>2371</v>
+        <v>2391</v>
       </c>
       <c r="B2095" s="2" t="s">
-        <v>2372</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="2096" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2096" s="2" t="s">
-        <v>2373</v>
+        <v>2393</v>
       </c>
       <c r="B2096" s="2" t="s">
-        <v>2374</v>
+        <v>2394</v>
       </c>
     </row>
     <row r="2097" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2097" s="2" t="s">
-        <v>2375</v>
-      </c>
-      <c r="B2097" s="2" t="s">
-        <v>2376</v>
+        <v>2395</v>
+      </c>
+      <c r="B2097" s="2" t="n">
+        <v>2193</v>
       </c>
     </row>
     <row r="2098" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2098" s="2" t="s">
-        <v>2377</v>
-      </c>
-      <c r="B2098" s="2" t="s">
-        <v>2378</v>
+        <v>2396</v>
+      </c>
+      <c r="B2098" s="2" t="n">
+        <v>2038</v>
       </c>
     </row>
     <row r="2099" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2099" s="2" t="s">
-        <v>2379</v>
-      </c>
-      <c r="B2099" s="2" t="s">
-        <v>2380</v>
+        <v>2397</v>
+      </c>
+      <c r="B2099" s="2" t="n">
+        <v>2039</v>
       </c>
     </row>
     <row r="2100" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2100" s="2" t="s">
-        <v>2381</v>
-      </c>
-      <c r="B2100" s="2" t="s">
-        <v>2382</v>
+        <v>2398</v>
+      </c>
+      <c r="B2100" s="2" t="n">
+        <v>2040</v>
       </c>
     </row>
     <row r="2101" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2101" s="2" t="s">
-        <v>2383</v>
+        <v>2399</v>
       </c>
       <c r="B2101" s="2" t="s">
-        <v>2384</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="2102" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2102" s="2" t="s">
-        <v>2385</v>
+        <v>2401</v>
       </c>
       <c r="B2102" s="2" t="s">
-        <v>2386</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="2103" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2103" s="2" t="s">
-        <v>2387</v>
+        <v>2403</v>
       </c>
       <c r="B2103" s="2" t="s">
-        <v>2388</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="2104" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2104" s="2" t="s">
-        <v>2389</v>
-      </c>
-      <c r="B2104" s="2" t="s">
-        <v>2390</v>
+        <v>2405</v>
+      </c>
+      <c r="B2104" s="2" t="n">
+        <v>1959</v>
       </c>
     </row>
     <row r="2105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2105" s="2" t="s">
-        <v>2391</v>
-      </c>
-      <c r="B2105" s="2" t="s">
-        <v>2392</v>
+        <v>2406</v>
+      </c>
+      <c r="B2105" s="2" t="n">
+        <v>2037</v>
       </c>
     </row>
     <row r="2106" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2106" s="2" t="s">
-        <v>2393</v>
-      </c>
-      <c r="B2106" s="2" t="s">
-        <v>2394</v>
+        <v>2407</v>
+      </c>
+      <c r="B2106" s="2" t="n">
+        <v>1958</v>
       </c>
     </row>
     <row r="2107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2107" s="2" t="s">
-        <v>2395</v>
-      </c>
-      <c r="B2107" s="2" t="s">
-        <v>2396</v>
+        <v>2408</v>
+      </c>
+      <c r="B2107" s="2" t="n">
+        <v>1904</v>
       </c>
     </row>
     <row r="2108" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2108" s="2" t="s">
-        <v>2397</v>
+        <v>2409</v>
       </c>
       <c r="B2108" s="2" t="s">
-        <v>2398</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="2109" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2109" s="2" t="s">
-        <v>2399</v>
-      </c>
-      <c r="B2109" s="2" t="s">
-        <v>2400</v>
+        <v>2410</v>
+      </c>
+      <c r="B2109" s="2" t="n">
+        <v>2194</v>
       </c>
     </row>
     <row r="2110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2110" s="2" t="s">
-        <v>2401</v>
+        <v>2411</v>
       </c>
       <c r="B2110" s="2" t="s">
-        <v>2402</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="2111" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2111" s="2" t="s">
-        <v>2403</v>
+        <v>2413</v>
       </c>
       <c r="B2111" s="2" t="s">
-        <v>2404</v>
+        <v>2414</v>
       </c>
     </row>
     <row r="2112" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2112" s="2" t="s">
-        <v>2405</v>
+        <v>2415</v>
       </c>
       <c r="B2112" s="2" t="s">
-        <v>2406</v>
+        <v>557</v>
       </c>
     </row>
     <row r="2113" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2113" s="2" t="s">
-        <v>2407</v>
-      </c>
-      <c r="B2113" s="2" t="s">
-        <v>2408</v>
+        <v>2416</v>
+      </c>
+      <c r="B2113" s="2" t="n">
+        <v>1863</v>
       </c>
     </row>
     <row r="2114" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2114" s="2" t="s">
-        <v>2409</v>
-      </c>
-      <c r="B2114" s="2" t="s">
-        <v>2410</v>
+        <v>2417</v>
+      </c>
+      <c r="B2114" s="2" t="n">
+        <v>2192</v>
       </c>
     </row>
     <row r="2115" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2115" s="2" t="s">
-        <v>2411</v>
-      </c>
-      <c r="B2115" s="2" t="s">
-        <v>2412</v>
+        <v>2418</v>
+      </c>
+      <c r="B2115" s="2" t="n">
+        <v>1859</v>
       </c>
     </row>
     <row r="2116" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2116" s="2" t="s">
-        <v>2413</v>
-      </c>
-      <c r="B2116" s="2" t="s">
-        <v>557</v>
+        <v>2419</v>
+      </c>
+      <c r="B2116" s="2" t="n">
+        <v>1860</v>
       </c>
     </row>
     <row r="2117" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2117" s="2" t="s">
-        <v>2414</v>
-      </c>
-      <c r="B2117" s="2" t="s">
-        <v>2415</v>
+        <v>2420</v>
+      </c>
+      <c r="B2117" s="2" t="n">
+        <v>1861</v>
       </c>
     </row>
     <row r="2118" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2118" s="2" t="s">
-        <v>2416</v>
+        <v>2421</v>
       </c>
       <c r="B2118" s="2" t="s">
-        <v>2417</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="2119" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2119" s="2" t="s">
-        <v>2418</v>
-      </c>
-      <c r="B2119" s="2" t="s">
-        <v>2419</v>
+        <v>2423</v>
+      </c>
+      <c r="B2119" s="2" t="n">
+        <v>1965</v>
       </c>
     </row>
     <row r="2120" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2120" s="2" t="s">
-        <v>2420</v>
-      </c>
-      <c r="B2120" s="2" t="s">
-        <v>2421</v>
+        <v>2424</v>
+      </c>
+      <c r="B2120" s="2" t="n">
+        <v>2255</v>
       </c>
     </row>
     <row r="2121" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2121" s="2" t="s">
-        <v>2422</v>
-      </c>
-      <c r="B2121" s="2" t="s">
-        <v>2423</v>
+        <v>2425</v>
+      </c>
+      <c r="B2121" s="2" t="n">
+        <v>1979</v>
       </c>
     </row>
     <row r="2122" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2122" s="2" t="s">
-        <v>2424</v>
-      </c>
-      <c r="B2122" s="2" t="s">
-        <v>2425</v>
+        <v>2426</v>
+      </c>
+      <c r="B2122" s="2" t="n">
+        <v>2013</v>
       </c>
     </row>
     <row r="2123" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2123" s="2" t="s">
-        <v>2426</v>
-      </c>
-      <c r="B2123" s="2" t="s">
         <v>2427</v>
+      </c>
+      <c r="B2123" s="2" t="n">
+        <v>2254</v>
       </c>
     </row>
     <row r="2124" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2124" s="2" t="s">
         <v>2428</v>
       </c>
-      <c r="B2124" s="2" t="s">
-        <v>2429</v>
+      <c r="B2124" s="2" t="n">
+        <v>1981</v>
       </c>
     </row>
     <row r="2125" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2125" s="2" t="s">
-        <v>2430</v>
-      </c>
-      <c r="B2125" s="2" t="s">
-        <v>2431</v>
+        <v>2429</v>
+      </c>
+      <c r="B2125" s="2" t="n">
+        <v>2253</v>
       </c>
     </row>
     <row r="2126" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2126" s="2" t="s">
-        <v>2432</v>
-      </c>
-      <c r="B2126" s="2" t="s">
-        <v>2433</v>
+        <v>2430</v>
+      </c>
+      <c r="B2126" s="2" t="n">
+        <v>2108</v>
       </c>
     </row>
     <row r="2127" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2127" s="2" t="s">
-        <v>2434</v>
+        <v>2431</v>
       </c>
       <c r="B2127" s="2" t="s">
-        <v>2435</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="2128" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2128" s="2" t="s">
-        <v>2436</v>
+        <v>2433</v>
       </c>
       <c r="B2128" s="2" t="s">
-        <v>2437</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="2129" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2129" s="2" t="s">
-        <v>2438</v>
+        <v>2435</v>
       </c>
       <c r="B2129" s="2" t="s">
-        <v>2439</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="2130" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2130" s="2" t="s">
-        <v>2440</v>
+        <v>2437</v>
       </c>
       <c r="B2130" s="2" t="s">
-        <v>2441</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="2131" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2131" s="2" t="s">
-        <v>2442</v>
+        <v>2439</v>
       </c>
       <c r="B2131" s="2" t="s">
-        <v>2443</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="2132" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2132" s="2" t="s">
-        <v>2444</v>
+        <v>2441</v>
       </c>
       <c r="B2132" s="2" t="s">
-        <v>2445</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="2133" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2133" s="2" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B2133" s="2" t="s">
+        <v>2444</v>
+      </c>
+    </row>
+    <row r="2134" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2134" s="2" t="s">
+        <v>2445</v>
+      </c>
+      <c r="B2134" s="2" t="n">
+        <v>1902</v>
+      </c>
+    </row>
+    <row r="2135" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2135" s="2" t="s">
         <v>2446</v>
       </c>
-      <c r="B2133" s="2" t="s">
+      <c r="B2135" s="2" t="n">
+        <v>1903</v>
+      </c>
+    </row>
+    <row r="2136" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2136" s="2" t="s">
         <v>2447</v>
+      </c>
+      <c r="B2136" s="2" t="s">
+        <v>2448</v>
+      </c>
+    </row>
+    <row r="2137" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2137" s="2" t="s">
+        <v>2449</v>
+      </c>
+      <c r="B2137" s="2" t="s">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="2138" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2138" s="2" t="s">
+        <v>2451</v>
+      </c>
+      <c r="B2138" s="2" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="2139" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2139" s="2" t="s">
+        <v>2453</v>
+      </c>
+      <c r="B2139" s="2" t="s">
+        <v>2454</v>
+      </c>
+    </row>
+    <row r="2140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2140" s="2" t="s">
+        <v>2455</v>
+      </c>
+      <c r="B2140" s="2" t="n">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="2141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2141" s="2" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B2141" s="2" t="s">
+        <v>2457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding M block parking updates
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2851" uniqueCount="2847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3011" uniqueCount="3007">
   <si>
     <t xml:space="preserve">Flat Number</t>
   </si>
@@ -8561,6 +8561,486 @@
   </si>
   <si>
     <t xml:space="preserve">L9-1204A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-702</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">764-765</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5-704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-307</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-306</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-1203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">716-717</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-1604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1206A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-1203A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-1101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-1603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B702</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5-503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-1407</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B714</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1203A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B715</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5-1603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B717</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-1202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B718</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B719</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5-701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B720</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B721</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B723</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5-1604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B724</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-1404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B726</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B727</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9-1204A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B728</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B729</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-1201A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B730</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B731</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2-1503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B732</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1206A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B733</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7-1205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B735</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3-206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B736</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1205A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B737</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B738</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B739</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B740</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7-1805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B743</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4-1202A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B744</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B745</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6-1601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">742-743</t>
   </si>
 </sst>
 </file>
@@ -8636,7 +9116,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -8647,6 +9127,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -8842,7 +9326,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B2565"/>
+  <dimension ref="A1:B2610"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12.63"/>
@@ -28785,296 +29269,948 @@
       </c>
     </row>
     <row r="2493" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2493" s="3"/>
-      <c r="B2493" s="3"/>
+      <c r="A2493" s="4" t="s">
+        <v>2847</v>
+      </c>
+      <c r="B2493" s="4" t="n">
+        <v>1603</v>
+      </c>
     </row>
     <row r="2494" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2494" s="3"/>
-      <c r="B2494" s="3"/>
+      <c r="A2494" s="4" t="s">
+        <v>2848</v>
+      </c>
+      <c r="B2494" s="4" t="n">
+        <v>1602</v>
+      </c>
     </row>
     <row r="2495" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2495" s="3"/>
-      <c r="B2495" s="3"/>
+      <c r="A2495" s="4" t="s">
+        <v>2849</v>
+      </c>
+      <c r="B2495" s="4" t="n">
+        <v>1601</v>
+      </c>
     </row>
     <row r="2496" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2496" s="3"/>
-      <c r="B2496" s="3"/>
+      <c r="A2496" s="4" t="s">
+        <v>2850</v>
+      </c>
+      <c r="B2496" s="4" t="n">
+        <v>1606</v>
+      </c>
     </row>
     <row r="2497" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2497" s="3"/>
-      <c r="B2497" s="3"/>
+      <c r="A2497" s="4" t="s">
+        <v>2851</v>
+      </c>
+      <c r="B2497" s="4" t="n">
+        <v>1609</v>
+      </c>
     </row>
     <row r="2498" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2498" s="3"/>
-      <c r="B2498" s="3"/>
+      <c r="A2498" s="4" t="s">
+        <v>2852</v>
+      </c>
+      <c r="B2498" s="4" t="n">
+        <v>1636</v>
+      </c>
     </row>
     <row r="2499" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2499" s="3"/>
-      <c r="B2499" s="3"/>
+      <c r="A2499" s="4" t="s">
+        <v>2853</v>
+      </c>
+      <c r="B2499" s="4" t="n">
+        <v>1632</v>
+      </c>
     </row>
     <row r="2500" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2500" s="3"/>
-      <c r="B2500" s="3"/>
+      <c r="A2500" s="4" t="s">
+        <v>2854</v>
+      </c>
+      <c r="B2500" s="4" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="2501" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2501" s="3"/>
-      <c r="B2501" s="3"/>
+      <c r="A2501" s="4" t="s">
+        <v>2855</v>
+      </c>
+      <c r="B2501" s="4" t="n">
+        <v>1645</v>
+      </c>
     </row>
     <row r="2502" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2502" s="3"/>
-      <c r="B2502" s="3"/>
+      <c r="A2502" s="4" t="s">
+        <v>2856</v>
+      </c>
+      <c r="B2502" s="4" t="n">
+        <v>1646</v>
+      </c>
     </row>
     <row r="2503" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2503" s="3"/>
-      <c r="B2503" s="3"/>
+      <c r="A2503" s="4" t="s">
+        <v>2857</v>
+      </c>
+      <c r="B2503" s="4" t="n">
+        <v>1673</v>
+      </c>
     </row>
     <row r="2504" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2504" s="3"/>
-      <c r="B2504" s="3"/>
+      <c r="A2504" s="4" t="s">
+        <v>2858</v>
+      </c>
+      <c r="B2504" s="4" t="s">
+        <v>2859</v>
+      </c>
     </row>
     <row r="2505" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2505" s="3"/>
-      <c r="B2505" s="3"/>
+      <c r="A2505" s="4" t="s">
+        <v>2860</v>
+      </c>
+      <c r="B2505" s="4" t="n">
+        <v>1669</v>
+      </c>
     </row>
     <row r="2506" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2506" s="3"/>
-      <c r="B2506" s="3"/>
+      <c r="A2506" s="4" t="s">
+        <v>2861</v>
+      </c>
+      <c r="B2506" s="4" t="n">
+        <v>1668</v>
+      </c>
     </row>
     <row r="2507" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2507" s="3"/>
-      <c r="B2507" s="3"/>
+      <c r="A2507" s="4" t="s">
+        <v>2862</v>
+      </c>
+      <c r="B2507" s="4" t="n">
+        <v>1667</v>
+      </c>
     </row>
     <row r="2508" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2508" s="3"/>
-      <c r="B2508" s="3"/>
+      <c r="A2508" s="4" t="s">
+        <v>2863</v>
+      </c>
+      <c r="B2508" s="4" t="n">
+        <v>1665</v>
+      </c>
     </row>
     <row r="2509" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2509" s="3"/>
-      <c r="B2509" s="3"/>
+      <c r="A2509" s="4" t="s">
+        <v>2864</v>
+      </c>
+      <c r="B2509" s="4" t="n">
+        <v>1657</v>
+      </c>
     </row>
     <row r="2510" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2510" s="3"/>
-      <c r="B2510" s="3"/>
+      <c r="A2510" s="4" t="s">
+        <v>2865</v>
+      </c>
+      <c r="B2510" s="4" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="2511" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2511" s="3"/>
-      <c r="B2511" s="3"/>
+      <c r="A2511" s="4" t="s">
+        <v>2866</v>
+      </c>
+      <c r="B2511" s="4" t="n">
+        <v>1683</v>
+      </c>
     </row>
     <row r="2512" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2512" s="3"/>
-      <c r="B2512" s="3"/>
+      <c r="A2512" s="4" t="s">
+        <v>2867</v>
+      </c>
+      <c r="B2512" s="4" t="n">
+        <v>1686</v>
+      </c>
     </row>
     <row r="2513" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2513" s="3"/>
-      <c r="B2513" s="3"/>
+      <c r="A2513" s="4" t="s">
+        <v>2868</v>
+      </c>
+      <c r="B2513" s="4" t="n">
+        <v>1687</v>
+      </c>
     </row>
     <row r="2514" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2514" s="3"/>
-      <c r="B2514" s="3"/>
+      <c r="A2514" s="4" t="s">
+        <v>2869</v>
+      </c>
+      <c r="B2514" s="4" t="n">
+        <v>1688</v>
+      </c>
     </row>
     <row r="2515" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2515" s="3"/>
-      <c r="B2515" s="3"/>
+      <c r="A2515" s="4" t="s">
+        <v>2870</v>
+      </c>
+      <c r="B2515" s="4" t="n">
+        <v>1689</v>
+      </c>
     </row>
     <row r="2516" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2516" s="3"/>
-      <c r="B2516" s="3"/>
+      <c r="A2516" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="B2516" s="4" t="n">
+        <v>1690</v>
+      </c>
     </row>
     <row r="2517" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2517" s="3"/>
-      <c r="B2517" s="3"/>
+      <c r="A2517" s="4" t="s">
+        <v>2872</v>
+      </c>
+      <c r="B2517" s="4" t="n">
+        <v>1694</v>
+      </c>
     </row>
     <row r="2518" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2518" s="3"/>
-      <c r="B2518" s="3"/>
+      <c r="A2518" s="4" t="s">
+        <v>2873</v>
+      </c>
+      <c r="B2518" s="4" t="n">
+        <v>1715</v>
+      </c>
     </row>
     <row r="2519" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2519" s="3"/>
-      <c r="B2519" s="3"/>
+      <c r="A2519" s="4" t="s">
+        <v>2874</v>
+      </c>
+      <c r="B2519" s="4" t="n">
+        <v>1712</v>
+      </c>
     </row>
     <row r="2520" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2520" s="3"/>
-      <c r="B2520" s="3"/>
+      <c r="A2520" s="4" t="s">
+        <v>2875</v>
+      </c>
+      <c r="B2520" s="4" t="n">
+        <v>1708</v>
+      </c>
     </row>
     <row r="2521" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2521" s="3"/>
-      <c r="B2521" s="3"/>
+      <c r="A2521" s="4" t="s">
+        <v>2876</v>
+      </c>
+      <c r="B2521" s="4" t="n">
+        <v>1699</v>
+      </c>
     </row>
     <row r="2522" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2522" s="3"/>
-      <c r="B2522" s="3"/>
+      <c r="A2522" s="4" t="s">
+        <v>2877</v>
+      </c>
+      <c r="B2522" s="4" t="n">
+        <v>1698</v>
+      </c>
     </row>
     <row r="2523" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2523" s="3"/>
-      <c r="B2523" s="3"/>
+      <c r="A2523" s="4" t="s">
+        <v>2878</v>
+      </c>
+      <c r="B2523" s="4" t="n">
+        <v>1731</v>
+      </c>
     </row>
     <row r="2524" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2524" s="3"/>
-      <c r="B2524" s="3"/>
+      <c r="A2524" s="4" t="s">
+        <v>2879</v>
+      </c>
+      <c r="B2524" s="4" t="n">
+        <v>1733</v>
+      </c>
     </row>
     <row r="2525" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2525" s="3"/>
-      <c r="B2525" s="3"/>
+      <c r="A2525" s="4" t="s">
+        <v>2880</v>
+      </c>
+      <c r="B2525" s="4" t="n">
+        <v>1734</v>
+      </c>
     </row>
     <row r="2526" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2526" s="3"/>
-      <c r="B2526" s="3"/>
+      <c r="A2526" s="4" t="s">
+        <v>2881</v>
+      </c>
+      <c r="B2526" s="4" t="n">
+        <v>1758</v>
+      </c>
     </row>
     <row r="2527" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2527" s="3"/>
-      <c r="B2527" s="3"/>
+      <c r="A2527" s="4" t="s">
+        <v>2882</v>
+      </c>
+      <c r="B2527" s="4" t="n">
+        <v>1736</v>
+      </c>
     </row>
     <row r="2528" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2528" s="3"/>
-      <c r="B2528" s="3"/>
+      <c r="A2528" s="4" t="s">
+        <v>2883</v>
+      </c>
+      <c r="B2528" s="4" t="n">
+        <v>1757</v>
+      </c>
     </row>
     <row r="2529" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2529" s="3"/>
-      <c r="B2529" s="3"/>
+      <c r="A2529" s="4" t="s">
+        <v>2884</v>
+      </c>
+      <c r="B2529" s="4" t="n">
+        <v>1755</v>
+      </c>
     </row>
     <row r="2530" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2530" s="3"/>
-      <c r="B2530" s="3"/>
+      <c r="A2530" s="4" t="s">
+        <v>2885</v>
+      </c>
+      <c r="B2530" s="4" t="n">
+        <v>1754</v>
+      </c>
     </row>
     <row r="2531" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2531" s="3"/>
-      <c r="B2531" s="3"/>
+      <c r="A2531" s="4" t="s">
+        <v>2886</v>
+      </c>
+      <c r="B2531" s="4" t="n">
+        <v>1753</v>
+      </c>
     </row>
     <row r="2532" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2532" s="3"/>
-      <c r="B2532" s="3"/>
+      <c r="A2532" s="4" t="s">
+        <v>2887</v>
+      </c>
+      <c r="B2532" s="4" t="n">
+        <v>1752</v>
+      </c>
     </row>
     <row r="2533" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2533" s="3"/>
-      <c r="B2533" s="3"/>
+      <c r="A2533" s="4" t="s">
+        <v>2888</v>
+      </c>
+      <c r="B2533" s="4" t="n">
+        <v>1749</v>
+      </c>
     </row>
     <row r="2534" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2534" s="3"/>
-      <c r="B2534" s="3"/>
+      <c r="A2534" s="4" t="s">
+        <v>2889</v>
+      </c>
+      <c r="B2534" s="4" t="n">
+        <v>1770</v>
+      </c>
     </row>
     <row r="2535" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2535" s="3"/>
-      <c r="B2535" s="3"/>
+      <c r="A2535" s="4" t="s">
+        <v>2890</v>
+      </c>
+      <c r="B2535" s="4" t="n">
+        <v>1780</v>
+      </c>
     </row>
     <row r="2536" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2536" s="3"/>
-      <c r="B2536" s="3"/>
+      <c r="A2536" s="4" t="s">
+        <v>2891</v>
+      </c>
+      <c r="B2536" s="4" t="n">
+        <v>1781</v>
+      </c>
     </row>
     <row r="2537" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2537" s="3"/>
-      <c r="B2537" s="3"/>
+      <c r="A2537" s="4" t="s">
+        <v>2892</v>
+      </c>
+      <c r="B2537" s="4" t="n">
+        <v>1782</v>
+      </c>
     </row>
     <row r="2538" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2538" s="3"/>
-      <c r="B2538" s="3"/>
+      <c r="A2538" s="4" t="s">
+        <v>2893</v>
+      </c>
+      <c r="B2538" s="4" t="n">
+        <v>1783</v>
+      </c>
     </row>
     <row r="2539" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2539" s="3"/>
-      <c r="B2539" s="3"/>
+      <c r="A2539" s="4" t="s">
+        <v>2894</v>
+      </c>
+      <c r="B2539" s="4" t="n">
+        <v>1784</v>
+      </c>
     </row>
     <row r="2540" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2540" s="3"/>
-      <c r="B2540" s="3"/>
+      <c r="A2540" s="4" t="s">
+        <v>2895</v>
+      </c>
+      <c r="B2540" s="4" t="n">
+        <v>1785</v>
+      </c>
     </row>
     <row r="2541" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2541" s="3"/>
-      <c r="B2541" s="3"/>
+      <c r="A2541" s="4" t="s">
+        <v>2896</v>
+      </c>
+      <c r="B2541" s="4" t="n">
+        <v>1786</v>
+      </c>
     </row>
     <row r="2542" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2542" s="3"/>
-      <c r="B2542" s="3"/>
+      <c r="A2542" s="4" t="s">
+        <v>2897</v>
+      </c>
+      <c r="B2542" s="4" t="n">
+        <v>1787</v>
+      </c>
     </row>
     <row r="2543" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2543" s="3"/>
-      <c r="B2543" s="3"/>
+      <c r="A2543" s="4" t="s">
+        <v>2898</v>
+      </c>
+      <c r="B2543" s="4" t="n">
+        <v>1788</v>
+      </c>
     </row>
     <row r="2544" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2544" s="3"/>
-      <c r="B2544" s="3"/>
+      <c r="A2544" s="4" t="s">
+        <v>2899</v>
+      </c>
+      <c r="B2544" s="4" t="n">
+        <v>1789</v>
+      </c>
     </row>
     <row r="2545" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2545" s="3"/>
-      <c r="B2545" s="3"/>
+      <c r="A2545" s="4" t="s">
+        <v>2900</v>
+      </c>
+      <c r="B2545" s="4" t="n">
+        <v>1794</v>
+      </c>
     </row>
     <row r="2546" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2546" s="3"/>
-      <c r="B2546" s="3"/>
+      <c r="A2546" s="4" t="s">
+        <v>2901</v>
+      </c>
+      <c r="B2546" s="4" t="n">
+        <v>1814</v>
+      </c>
     </row>
     <row r="2547" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2547" s="3"/>
-      <c r="B2547" s="3"/>
+      <c r="A2547" s="4" t="s">
+        <v>2902</v>
+      </c>
+      <c r="B2547" s="4" t="s">
+        <v>2903</v>
+      </c>
     </row>
     <row r="2548" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2548" s="3"/>
-      <c r="B2548" s="3"/>
+      <c r="A2548" s="4" t="s">
+        <v>2904</v>
+      </c>
+      <c r="B2548" s="4" t="n">
+        <v>1813</v>
+      </c>
     </row>
     <row r="2549" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2549" s="3"/>
-      <c r="B2549" s="3"/>
+      <c r="A2549" s="4" t="s">
+        <v>2905</v>
+      </c>
+      <c r="B2549" s="4" t="n">
+        <v>1812</v>
+      </c>
     </row>
     <row r="2550" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2550" s="3"/>
-      <c r="B2550" s="3"/>
+      <c r="A2550" s="4" t="s">
+        <v>2906</v>
+      </c>
+      <c r="B2550" s="4" t="n">
+        <v>1810</v>
+      </c>
     </row>
     <row r="2551" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2551" s="3"/>
-      <c r="B2551" s="3"/>
+      <c r="A2551" s="4" t="s">
+        <v>2907</v>
+      </c>
+      <c r="B2551" s="4" t="n">
+        <v>1808</v>
+      </c>
     </row>
     <row r="2552" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2552" s="3"/>
-      <c r="B2552" s="3"/>
+      <c r="A2552" s="4" t="s">
+        <v>2908</v>
+      </c>
+      <c r="B2552" s="4" t="n">
+        <v>1807</v>
+      </c>
     </row>
     <row r="2553" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2553" s="3"/>
-      <c r="B2553" s="3"/>
+      <c r="A2553" s="4" t="s">
+        <v>2909</v>
+      </c>
+      <c r="B2553" s="4" t="n">
+        <v>1806</v>
+      </c>
     </row>
     <row r="2554" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2554" s="3"/>
-      <c r="B2554" s="3"/>
+      <c r="A2554" s="4" t="s">
+        <v>2910</v>
+      </c>
+      <c r="B2554" s="4" t="n">
+        <v>1805</v>
+      </c>
     </row>
     <row r="2555" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2555" s="3"/>
-      <c r="B2555" s="3"/>
+      <c r="A2555" s="4" t="s">
+        <v>2911</v>
+      </c>
+      <c r="B2555" s="4" t="n">
+        <v>1804</v>
+      </c>
     </row>
     <row r="2556" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2556" s="3"/>
-      <c r="B2556" s="3"/>
+      <c r="A2556" s="4" t="s">
+        <v>2912</v>
+      </c>
+      <c r="B2556" s="4" t="n">
+        <v>1799</v>
+      </c>
     </row>
     <row r="2557" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2557" s="3"/>
-      <c r="B2557" s="3"/>
+      <c r="A2557" s="4" t="s">
+        <v>2913</v>
+      </c>
+      <c r="B2557" s="4" t="n">
+        <v>1829</v>
+      </c>
     </row>
     <row r="2558" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2558" s="3"/>
-      <c r="B2558" s="3"/>
+      <c r="A2558" s="4" t="s">
+        <v>2914</v>
+      </c>
+      <c r="B2558" s="4" t="n">
+        <v>1837</v>
+      </c>
     </row>
     <row r="2559" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2559" s="3"/>
-      <c r="B2559" s="3"/>
+      <c r="A2559" s="4" t="s">
+        <v>2915</v>
+      </c>
+      <c r="B2559" s="4" t="n">
+        <v>1838</v>
+      </c>
     </row>
     <row r="2560" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2560" s="3"/>
-      <c r="B2560" s="3"/>
+      <c r="A2560" s="4" t="s">
+        <v>2916</v>
+      </c>
+      <c r="B2560" s="4" t="n">
+        <v>1839</v>
+      </c>
     </row>
     <row r="2561" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2561" s="3"/>
-      <c r="B2561" s="3"/>
+      <c r="A2561" s="4" t="s">
+        <v>2917</v>
+      </c>
+      <c r="B2561" s="4" t="n">
+        <v>1840</v>
+      </c>
     </row>
     <row r="2562" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2562" s="3"/>
-      <c r="B2562" s="3"/>
+      <c r="A2562" s="4" t="s">
+        <v>2918</v>
+      </c>
+      <c r="B2562" s="4" t="n">
+        <v>1841</v>
+      </c>
     </row>
     <row r="2563" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2563" s="3"/>
-      <c r="B2563" s="3"/>
+      <c r="A2563" s="4" t="s">
+        <v>2919</v>
+      </c>
+      <c r="B2563" s="4" t="n">
+        <v>1842</v>
+      </c>
     </row>
     <row r="2564" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2564" s="3"/>
-      <c r="B2564" s="3"/>
+      <c r="A2564" s="4" t="s">
+        <v>2920</v>
+      </c>
+      <c r="B2564" s="4" t="n">
+        <v>1843</v>
+      </c>
     </row>
     <row r="2565" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2565" s="3"/>
-      <c r="B2565" s="3"/>
+      <c r="A2565" s="4" t="s">
+        <v>2921</v>
+      </c>
+      <c r="B2565" s="4" t="n">
+        <v>1844</v>
+      </c>
+    </row>
+    <row r="2566" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2566" s="4" t="s">
+        <v>2922</v>
+      </c>
+      <c r="B2566" s="4" t="n">
+        <v>1845</v>
+      </c>
+    </row>
+    <row r="2567" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2567" s="4" t="s">
+        <v>2923</v>
+      </c>
+      <c r="B2567" s="4" t="n">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="2568" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2568" s="4" t="s">
+        <v>2924</v>
+      </c>
+      <c r="B2568" s="4" t="n">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="2569" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2569" s="4" t="s">
+        <v>2925</v>
+      </c>
+      <c r="B2569" s="4" t="n">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="2570" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2570" s="4" t="s">
+        <v>2926</v>
+      </c>
+      <c r="B2570" s="4" t="s">
+        <v>2927</v>
+      </c>
+    </row>
+    <row r="2571" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2571" s="4" t="s">
+        <v>2928</v>
+      </c>
+      <c r="B2571" s="4" t="s">
+        <v>2929</v>
+      </c>
+    </row>
+    <row r="2572" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2572" s="4" t="s">
+        <v>2930</v>
+      </c>
+      <c r="B2572" s="4" t="n">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="2573" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2573" s="4" t="s">
+        <v>2931</v>
+      </c>
+      <c r="B2573" s="4" t="s">
+        <v>2932</v>
+      </c>
+    </row>
+    <row r="2574" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2574" s="4" t="s">
+        <v>2933</v>
+      </c>
+      <c r="B2574" s="4" t="s">
+        <v>2934</v>
+      </c>
+    </row>
+    <row r="2575" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2575" s="4" t="s">
+        <v>2935</v>
+      </c>
+      <c r="B2575" s="4" t="s">
+        <v>2936</v>
+      </c>
+    </row>
+    <row r="2576" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2576" s="4" t="s">
+        <v>2937</v>
+      </c>
+      <c r="B2576" s="4" t="s">
+        <v>2938</v>
+      </c>
+    </row>
+    <row r="2577" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2577" s="4" t="s">
+        <v>2939</v>
+      </c>
+      <c r="B2577" s="4" t="s">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="2578" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2578" s="4" t="s">
+        <v>2941</v>
+      </c>
+      <c r="B2578" s="4" t="s">
+        <v>2942</v>
+      </c>
+    </row>
+    <row r="2579" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2579" s="4" t="s">
+        <v>2943</v>
+      </c>
+      <c r="B2579" s="4" t="s">
+        <v>2944</v>
+      </c>
+    </row>
+    <row r="2580" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2580" s="4" t="s">
+        <v>2945</v>
+      </c>
+      <c r="B2580" s="4" t="s">
+        <v>2946</v>
+      </c>
+    </row>
+    <row r="2581" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2581" s="4" t="s">
+        <v>2947</v>
+      </c>
+      <c r="B2581" s="4" t="s">
+        <v>2948</v>
+      </c>
+    </row>
+    <row r="2582" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2582" s="4" t="s">
+        <v>2949</v>
+      </c>
+      <c r="B2582" s="4" t="s">
+        <v>2950</v>
+      </c>
+    </row>
+    <row r="2583" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2583" s="4" t="s">
+        <v>2951</v>
+      </c>
+      <c r="B2583" s="4" t="s">
+        <v>2952</v>
+      </c>
+    </row>
+    <row r="2584" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2584" s="4" t="s">
+        <v>2953</v>
+      </c>
+      <c r="B2584" s="4" t="s">
+        <v>2954</v>
+      </c>
+    </row>
+    <row r="2585" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2585" s="4" t="s">
+        <v>2955</v>
+      </c>
+      <c r="B2585" s="4" t="s">
+        <v>2956</v>
+      </c>
+    </row>
+    <row r="2586" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2586" s="4" t="s">
+        <v>2957</v>
+      </c>
+      <c r="B2586" s="4" t="s">
+        <v>2958</v>
+      </c>
+    </row>
+    <row r="2587" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2587" s="4" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B2587" s="4" t="s">
+        <v>2960</v>
+      </c>
+    </row>
+    <row r="2588" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2588" s="4" t="s">
+        <v>2961</v>
+      </c>
+      <c r="B2588" s="4" t="s">
+        <v>2962</v>
+      </c>
+    </row>
+    <row r="2589" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2589" s="4" t="s">
+        <v>2963</v>
+      </c>
+      <c r="B2589" s="4" t="s">
+        <v>2964</v>
+      </c>
+    </row>
+    <row r="2590" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2590" s="4" t="s">
+        <v>2965</v>
+      </c>
+      <c r="B2590" s="4" t="s">
+        <v>2966</v>
+      </c>
+    </row>
+    <row r="2591" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2591" s="4" t="s">
+        <v>2967</v>
+      </c>
+      <c r="B2591" s="4" t="s">
+        <v>2968</v>
+      </c>
+    </row>
+    <row r="2592" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2592" s="4" t="s">
+        <v>2969</v>
+      </c>
+      <c r="B2592" s="4" t="s">
+        <v>2970</v>
+      </c>
+    </row>
+    <row r="2593" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2593" s="4" t="s">
+        <v>2971</v>
+      </c>
+      <c r="B2593" s="4" t="s">
+        <v>2972</v>
+      </c>
+    </row>
+    <row r="2594" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2594" s="4" t="s">
+        <v>2973</v>
+      </c>
+      <c r="B2594" s="4" t="s">
+        <v>2974</v>
+      </c>
+    </row>
+    <row r="2595" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2595" s="4" t="s">
+        <v>2975</v>
+      </c>
+      <c r="B2595" s="4" t="s">
+        <v>2976</v>
+      </c>
+    </row>
+    <row r="2596" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2596" s="4" t="s">
+        <v>2977</v>
+      </c>
+      <c r="B2596" s="4" t="s">
+        <v>2978</v>
+      </c>
+    </row>
+    <row r="2597" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2597" s="4" t="s">
+        <v>2979</v>
+      </c>
+      <c r="B2597" s="4" t="s">
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="2598" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2598" s="4" t="s">
+        <v>2981</v>
+      </c>
+      <c r="B2598" s="4" t="s">
+        <v>2982</v>
+      </c>
+    </row>
+    <row r="2599" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2599" s="4" t="s">
+        <v>2983</v>
+      </c>
+      <c r="B2599" s="4" t="s">
+        <v>2984</v>
+      </c>
+    </row>
+    <row r="2600" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2600" s="4" t="s">
+        <v>2985</v>
+      </c>
+      <c r="B2600" s="4" t="s">
+        <v>2986</v>
+      </c>
+    </row>
+    <row r="2601" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2601" s="4" t="s">
+        <v>2987</v>
+      </c>
+      <c r="B2601" s="4" t="s">
+        <v>2988</v>
+      </c>
+    </row>
+    <row r="2602" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2602" s="4" t="s">
+        <v>2989</v>
+      </c>
+      <c r="B2602" s="4" t="s">
+        <v>2990</v>
+      </c>
+    </row>
+    <row r="2603" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2603" s="4" t="s">
+        <v>2991</v>
+      </c>
+      <c r="B2603" s="4" t="s">
+        <v>2992</v>
+      </c>
+    </row>
+    <row r="2604" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2604" s="4" t="s">
+        <v>2993</v>
+      </c>
+      <c r="B2604" s="4" t="s">
+        <v>2994</v>
+      </c>
+    </row>
+    <row r="2605" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2605" s="4" t="s">
+        <v>2995</v>
+      </c>
+      <c r="B2605" s="4" t="s">
+        <v>2996</v>
+      </c>
+    </row>
+    <row r="2606" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2606" s="4" t="s">
+        <v>2997</v>
+      </c>
+      <c r="B2606" s="4" t="s">
+        <v>2998</v>
+      </c>
+    </row>
+    <row r="2607" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2607" s="4" t="s">
+        <v>2999</v>
+      </c>
+      <c r="B2607" s="4" t="s">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="2608" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2608" s="4" t="s">
+        <v>3001</v>
+      </c>
+      <c r="B2608" s="4" t="s">
+        <v>3002</v>
+      </c>
+    </row>
+    <row r="2609" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2609" s="4" t="s">
+        <v>3003</v>
+      </c>
+      <c r="B2609" s="4" t="s">
+        <v>3004</v>
+      </c>
+    </row>
+    <row r="2610" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2610" s="4" t="s">
+        <v>3005</v>
+      </c>
+      <c r="B2610" s="4" t="s">
+        <v>3006</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Mutual swap 500 & 578
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9573,7 +9573,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -16162,7 +16162,7 @@
         <v>1035</v>
       </c>
       <c r="B796" s="3" t="n">
-        <v>578</v>
+        <v>500</v>
       </c>
     </row>
     <row r="797" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17090,7 +17090,7 @@
         <v>1170</v>
       </c>
       <c r="B912" s="3" t="n">
-        <v>500</v>
+        <v>578</v>
       </c>
     </row>
     <row r="913" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
adding J block new parkings
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3156" uniqueCount="3154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3223" uniqueCount="3221">
   <si>
     <t xml:space="preserve">Flat Number</t>
   </si>
@@ -7993,7 +7993,7 @@
     <t xml:space="preserve">M5-503</t>
   </si>
   <si>
-    <t xml:space="preserve">B705</t>
+    <t xml:space="preserve">B785</t>
   </si>
   <si>
     <t xml:space="preserve">M5-603</t>
@@ -9485,6 +9485,207 @@
   </si>
   <si>
     <t xml:space="preserve">M7-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4-105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-495</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J8-1205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-587</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-542</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1-1903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-639</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2-1901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-644</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1-904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-567</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4-701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-633</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1-1204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-543</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1-1203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-529</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5-404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-635</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J8-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2-1801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-611</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4-1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-520</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-694</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2-401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-612</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-596</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7-1205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-696</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2-304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-562</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7-1805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-695</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7-501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-511</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8-1205A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-702</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4-302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-654</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J8-1406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-521</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-1202A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-682</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J8-1701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-586</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-575</t>
   </si>
 </sst>
 </file>
@@ -9573,7 +9774,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -16162,7 +16363,7 @@
         <v>1035</v>
       </c>
       <c r="B796" s="3" t="n">
-        <v>500</v>
+        <v>578</v>
       </c>
     </row>
     <row r="797" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17090,7 +17291,7 @@
         <v>1170</v>
       </c>
       <c r="B912" s="3" t="n">
-        <v>578</v>
+        <v>500</v>
       </c>
     </row>
     <row r="913" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31310,140 +31511,276 @@
       </c>
     </row>
     <row r="2690" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2690" s="4"/>
-      <c r="B2690" s="4"/>
+      <c r="A2690" s="3" t="s">
+        <v>3154</v>
+      </c>
+      <c r="B2690" s="3" t="n">
+        <v>534</v>
+      </c>
     </row>
     <row r="2691" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2691" s="4"/>
-      <c r="B2691" s="4"/>
+      <c r="A2691" s="3" t="s">
+        <v>3155</v>
+      </c>
+      <c r="B2691" s="3" t="s">
+        <v>3156</v>
+      </c>
     </row>
     <row r="2692" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2692" s="4"/>
-      <c r="B2692" s="4"/>
+      <c r="A2692" s="3" t="s">
+        <v>3157</v>
+      </c>
+      <c r="B2692" s="3" t="s">
+        <v>3158</v>
+      </c>
     </row>
     <row r="2693" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2693" s="4"/>
-      <c r="B2693" s="4"/>
+      <c r="A2693" s="3" t="s">
+        <v>3159</v>
+      </c>
+      <c r="B2693" s="3" t="s">
+        <v>3160</v>
+      </c>
     </row>
     <row r="2694" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2694" s="4"/>
-      <c r="B2694" s="4"/>
+      <c r="A2694" s="3" t="s">
+        <v>3161</v>
+      </c>
+      <c r="B2694" s="3" t="s">
+        <v>3162</v>
+      </c>
     </row>
     <row r="2695" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2695" s="4"/>
-      <c r="B2695" s="4"/>
+      <c r="A2695" s="3" t="s">
+        <v>3163</v>
+      </c>
+      <c r="B2695" s="3" t="s">
+        <v>3164</v>
+      </c>
     </row>
     <row r="2696" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2696" s="4"/>
-      <c r="B2696" s="4"/>
+      <c r="A2696" s="3" t="s">
+        <v>3165</v>
+      </c>
+      <c r="B2696" s="3" t="s">
+        <v>3166</v>
+      </c>
     </row>
     <row r="2697" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2697" s="4"/>
-      <c r="B2697" s="4"/>
+      <c r="A2697" s="3" t="s">
+        <v>3167</v>
+      </c>
+      <c r="B2697" s="3" t="s">
+        <v>3168</v>
+      </c>
     </row>
     <row r="2698" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2698" s="4"/>
-      <c r="B2698" s="4"/>
+      <c r="A2698" s="3" t="s">
+        <v>3169</v>
+      </c>
+      <c r="B2698" s="3" t="s">
+        <v>3170</v>
+      </c>
     </row>
     <row r="2699" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2699" s="4"/>
-      <c r="B2699" s="4"/>
+      <c r="A2699" s="3" t="s">
+        <v>3171</v>
+      </c>
+      <c r="B2699" s="3" t="s">
+        <v>3172</v>
+      </c>
     </row>
     <row r="2700" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2700" s="4"/>
-      <c r="B2700" s="4"/>
+      <c r="A2700" s="3" t="s">
+        <v>3173</v>
+      </c>
+      <c r="B2700" s="3" t="s">
+        <v>3174</v>
+      </c>
     </row>
     <row r="2701" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2701" s="4"/>
-      <c r="B2701" s="4"/>
+      <c r="A2701" s="3" t="s">
+        <v>3175</v>
+      </c>
+      <c r="B2701" s="3" t="s">
+        <v>3176</v>
+      </c>
     </row>
     <row r="2702" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2702" s="4"/>
-      <c r="B2702" s="4"/>
+      <c r="A2702" s="3" t="s">
+        <v>3177</v>
+      </c>
+      <c r="B2702" s="3" t="s">
+        <v>3178</v>
+      </c>
     </row>
     <row r="2703" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2703" s="4"/>
-      <c r="B2703" s="4"/>
+      <c r="A2703" s="3" t="s">
+        <v>3179</v>
+      </c>
+      <c r="B2703" s="3" t="s">
+        <v>3180</v>
+      </c>
     </row>
     <row r="2704" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2704" s="4"/>
-      <c r="B2704" s="4"/>
+      <c r="A2704" s="3" t="s">
+        <v>3181</v>
+      </c>
+      <c r="B2704" s="3" t="s">
+        <v>3182</v>
+      </c>
     </row>
     <row r="2705" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2705" s="4"/>
-      <c r="B2705" s="4"/>
+      <c r="A2705" s="3" t="s">
+        <v>3183</v>
+      </c>
+      <c r="B2705" s="3" t="s">
+        <v>3184</v>
+      </c>
     </row>
     <row r="2706" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2706" s="4"/>
-      <c r="B2706" s="4"/>
+      <c r="A2706" s="3" t="s">
+        <v>3185</v>
+      </c>
+      <c r="B2706" s="3" t="s">
+        <v>3186</v>
+      </c>
     </row>
     <row r="2707" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2707" s="4"/>
-      <c r="B2707" s="4"/>
+      <c r="A2707" s="3" t="s">
+        <v>3187</v>
+      </c>
+      <c r="B2707" s="3" t="s">
+        <v>3188</v>
+      </c>
     </row>
     <row r="2708" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2708" s="4"/>
-      <c r="B2708" s="4"/>
+      <c r="A2708" s="3" t="s">
+        <v>3189</v>
+      </c>
+      <c r="B2708" s="3" t="s">
+        <v>3190</v>
+      </c>
     </row>
     <row r="2709" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2709" s="4"/>
-      <c r="B2709" s="4"/>
+      <c r="A2709" s="3" t="s">
+        <v>3191</v>
+      </c>
+      <c r="B2709" s="3" t="s">
+        <v>3192</v>
+      </c>
     </row>
     <row r="2710" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2710" s="4"/>
-      <c r="B2710" s="4"/>
+      <c r="A2710" s="3" t="s">
+        <v>3193</v>
+      </c>
+      <c r="B2710" s="3" t="s">
+        <v>3194</v>
+      </c>
     </row>
     <row r="2711" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2711" s="4"/>
-      <c r="B2711" s="4"/>
+      <c r="A2711" s="3" t="s">
+        <v>3195</v>
+      </c>
+      <c r="B2711" s="3" t="s">
+        <v>3196</v>
+      </c>
     </row>
     <row r="2712" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2712" s="4"/>
-      <c r="B2712" s="4"/>
+      <c r="A2712" s="3" t="s">
+        <v>3197</v>
+      </c>
+      <c r="B2712" s="3" t="s">
+        <v>3198</v>
+      </c>
     </row>
     <row r="2713" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2713" s="4"/>
-      <c r="B2713" s="4"/>
+      <c r="A2713" s="3" t="s">
+        <v>3199</v>
+      </c>
+      <c r="B2713" s="3" t="s">
+        <v>3200</v>
+      </c>
     </row>
     <row r="2714" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2714" s="4"/>
-      <c r="B2714" s="4"/>
+      <c r="A2714" s="3" t="s">
+        <v>3201</v>
+      </c>
+      <c r="B2714" s="3" t="s">
+        <v>3202</v>
+      </c>
     </row>
     <row r="2715" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2715" s="4"/>
-      <c r="B2715" s="4"/>
+      <c r="A2715" s="3" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B2715" s="3" t="s">
+        <v>3204</v>
+      </c>
     </row>
     <row r="2716" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2716" s="4"/>
-      <c r="B2716" s="4"/>
+      <c r="A2716" s="3" t="s">
+        <v>3205</v>
+      </c>
+      <c r="B2716" s="3" t="s">
+        <v>3206</v>
+      </c>
     </row>
     <row r="2717" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2717" s="4"/>
-      <c r="B2717" s="4"/>
+      <c r="A2717" s="3" t="s">
+        <v>3207</v>
+      </c>
+      <c r="B2717" s="3" t="s">
+        <v>3208</v>
+      </c>
     </row>
     <row r="2718" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2718" s="4"/>
-      <c r="B2718" s="4"/>
+      <c r="A2718" s="3" t="s">
+        <v>3209</v>
+      </c>
+      <c r="B2718" s="3" t="s">
+        <v>3210</v>
+      </c>
     </row>
     <row r="2719" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2719" s="4"/>
-      <c r="B2719" s="4"/>
+      <c r="A2719" s="3" t="s">
+        <v>3211</v>
+      </c>
+      <c r="B2719" s="3" t="s">
+        <v>3212</v>
+      </c>
     </row>
     <row r="2720" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2720" s="4"/>
-      <c r="B2720" s="4"/>
+      <c r="A2720" s="3" t="s">
+        <v>3213</v>
+      </c>
+      <c r="B2720" s="3" t="s">
+        <v>3214</v>
+      </c>
     </row>
     <row r="2721" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2721" s="4"/>
-      <c r="B2721" s="4"/>
+      <c r="A2721" s="3" t="s">
+        <v>3215</v>
+      </c>
+      <c r="B2721" s="3" t="s">
+        <v>3216</v>
+      </c>
     </row>
     <row r="2722" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2722" s="4"/>
-      <c r="B2722" s="4"/>
+      <c r="A2722" s="3" t="s">
+        <v>3217</v>
+      </c>
+      <c r="B2722" s="3" t="s">
+        <v>3218</v>
+      </c>
     </row>
     <row r="2723" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2723" s="4"/>
-      <c r="B2723" s="4"/>
+      <c r="A2723" s="3" t="s">
+        <v>3219</v>
+      </c>
+      <c r="B2723" s="3" t="s">
+        <v>3220</v>
+      </c>
     </row>
     <row r="2724" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2724" s="4"/>

</xml_diff>

<commit_message>
adding M block parkin details
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3223" uniqueCount="3221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3225" uniqueCount="3223">
   <si>
     <t xml:space="preserve">Flat Number</t>
   </si>
@@ -7468,7 +7468,7 @@
     <t xml:space="preserve">M2-1503</t>
   </si>
   <si>
-    <t xml:space="preserve">B732</t>
+    <t xml:space="preserve">689-690</t>
   </si>
   <si>
     <t xml:space="preserve">M2-1603</t>
@@ -8059,7 +8059,7 @@
     <t xml:space="preserve">M6-1501</t>
   </si>
   <si>
-    <t xml:space="preserve">712A</t>
+    <t xml:space="preserve">812A</t>
   </si>
   <si>
     <t xml:space="preserve">M6-1504</t>
@@ -9686,6 +9686,12 @@
   </si>
   <si>
     <t xml:space="preserve">B-575</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1-1504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">662-663</t>
   </si>
 </sst>
 </file>
@@ -9774,7 +9780,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -28059,7 +28065,7 @@
         <v>2716</v>
       </c>
       <c r="B2258" s="3" t="n">
-        <v>633</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2259" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31783,8 +31789,12 @@
       </c>
     </row>
     <row r="2724" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2724" s="4"/>
-      <c r="B2724" s="4"/>
+      <c r="A2724" s="4" t="s">
+        <v>3221</v>
+      </c>
+      <c r="B2724" s="4" t="s">
+        <v>3222</v>
+      </c>
     </row>
     <row r="2725" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2725" s="4"/>

</xml_diff>